<commit_message>
Mark PR-01 done in the delivery plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="378">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #1</t>
   </si>
   <si>
     <t xml:space="preserve">PR-02</t>
@@ -321,6 +321,12 @@
   </si>
   <si>
     <t xml:space="preserve">Invariants in the schema not the app; why tool_calls separate from messages; HNSW vs IVFFlat; denormalised business_id on chunks; one conversation per session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design doc reviewed and merged first (PR #2, docs/database-design.md)</t>
   </si>
   <si>
     <t xml:space="preserve">PR-03</t>
@@ -1523,24 +1529,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1572,7 +1582,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1584,11 +1594,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1596,51 +1606,51 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1733,7 +1743,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="26">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -1759,6 +1769,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9CA3AF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1855,6 +1873,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF0000FF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFBBF7D0"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2243,456 +2269,456 @@
   <dimension ref="A1:E43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <f aca="false">COUNTA('PR Plan'!$A$5:$A$18)</f>
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"In progress")+COUNTIF('PR Plan'!$M$5:$M$18,"In review")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <f aca="false">SUM('PR Plan'!$K$5:$K$18)</f>
         <v>27</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+        <v>0.0185185185185185</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <f aca="false">COUNTA('Story Coverage'!$A$5:$A$1000)</f>
         <v>49</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$D:$D,"Must")</f>
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$L$5:$L$18,A18)</f>
         <v>8.5</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">B18-C18</f>
         <v>-0.5</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$18,A18)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$L$5:$L$18,A19)</f>
         <v>11.5</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">B19-C19</f>
         <v>0.5</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$18,A19)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$L$5:$L$18,A20)</f>
         <v>5</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="11" t="n">
         <f aca="false">B20-C20</f>
         <v>0</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$18,A20)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$L$5:$L$18,A21)</f>
         <v>2</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">B21-C21</f>
         <v>-2</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$18,A21)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="14" t="n">
         <f aca="false">SUM(B18:B21)</f>
         <v>25</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="14" t="n">
         <f aca="false">SUM(C18:C21)</f>
         <v>27</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="14" t="n">
         <f aca="false">B22-C22</f>
         <v>-2</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">SUM(E18:E21)</f>
         <v>14</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A27)</f>
         <v>2.5</v>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A27)</f>
         <v>3</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A27,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A28)</f>
         <v>3.5</v>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A28)</f>
         <v>2</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A28,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A29)</f>
         <v>5</v>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A29)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A29,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A30)</f>
         <v>3</v>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C30" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A30)</f>
         <v>1</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A30,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A31)</f>
         <v>4</v>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C31" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A31)</f>
         <v>1</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A31,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A32)</f>
         <v>5.5</v>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C32" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A32)</f>
         <v>3</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A32,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A33)</f>
         <v>1.5</v>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A33)</f>
         <v>1</v>
       </c>
-      <c r="D33" s="17" t="n">
+      <c r="D33" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A33,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="24" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="10" t="n">
+      <c r="B34" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$D$5:$D$18,A34)</f>
         <v>2</v>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C34" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$18,A34)</f>
         <v>1</v>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D34" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A34,'PR Plan'!$M$5:$M$18,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="27" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="27" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" s="27" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="27" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="27" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" s="27" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" s="27" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="27" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2721,779 +2747,783 @@
   <dimension ref="A1:O20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="G4" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="H4" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="I4" s="30" t="s">
+      <c r="I4" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="J4" s="30" t="s">
+      <c r="J4" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="K4" s="30" t="s">
+      <c r="K4" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="30" t="s">
+      <c r="L4" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="M4" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="N4" s="30" t="s">
+      <c r="N4" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="O4" s="30" t="s">
+      <c r="O4" s="31" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="I5" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="34" t="s">
+      <c r="J5" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="K5" s="35" t="n">
+      <c r="K5" s="36" t="n">
         <v>0.5</v>
       </c>
-      <c r="L5" s="34" t="s">
+      <c r="L5" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N5" s="34" t="n">
+      <c r="M5" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="N5" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A5)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="37"/>
+      <c r="O5" s="38" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="J6" s="34" t="s">
+      <c r="J6" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="K6" s="35" t="n">
+      <c r="K6" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L6" s="34" t="s">
+      <c r="L6" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N6" s="34" t="n">
+      <c r="M6" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N6" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A6)</f>
         <v>1</v>
       </c>
-      <c r="O6" s="37"/>
+      <c r="O6" s="38" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="J7" s="35" t="s">
+        <v>79</v>
+      </c>
+      <c r="K7" s="36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L7" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="M7" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="32" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="32" t="s">
-        <v>91</v>
-      </c>
-      <c r="I7" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="J7" s="34" t="s">
-        <v>79</v>
-      </c>
-      <c r="K7" s="35" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="L7" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="M7" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N7" s="34" t="n">
+      <c r="N7" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A7)</f>
         <v>0</v>
       </c>
-      <c r="O7" s="37"/>
+      <c r="O7" s="38"/>
     </row>
     <row r="8" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="32" t="s">
+      <c r="A8" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="B8" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="G8" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="H8" s="32" t="s">
+      <c r="F8" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="G8" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="H8" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="J8" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="K8" s="35" t="n">
+      <c r="K8" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="L8" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N8" s="34" t="n">
+      <c r="M8" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N8" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A8)</f>
         <v>2</v>
       </c>
-      <c r="O8" s="37"/>
+      <c r="O8" s="38"/>
     </row>
     <row r="9" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="C9" s="32" t="s">
+      <c r="A9" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="B9" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="34" t="s">
+      <c r="E9" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="32" t="s">
-        <v>103</v>
-      </c>
-      <c r="G9" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="H9" s="32" t="s">
+      <c r="F9" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="G9" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="J9" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="K9" s="35" t="n">
+      <c r="H9" s="33" t="s">
+        <v>107</v>
+      </c>
+      <c r="I9" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="J9" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L9" s="34" t="s">
+      <c r="L9" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N9" s="34" t="n">
+      <c r="M9" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
         <v>3</v>
       </c>
-      <c r="O9" s="37"/>
+      <c r="O9" s="38"/>
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="32" t="s">
+      <c r="A10" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="B10" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" s="32" t="s">
-        <v>111</v>
-      </c>
-      <c r="H10" s="32" t="s">
+      <c r="F10" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="I10" s="32" t="s">
+      <c r="G10" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="J10" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="K10" s="35" t="n">
+      <c r="H10" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="I10" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="J10" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="K10" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="L10" s="34" t="s">
+      <c r="L10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M10" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N10" s="34" t="n">
+      <c r="M10" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
         <v>11</v>
       </c>
-      <c r="O10" s="37"/>
+      <c r="O10" s="38"/>
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
-        <v>114</v>
-      </c>
-      <c r="B11" s="32" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" s="32" t="s">
+      <c r="A11" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="B11" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="32" t="s">
-        <v>117</v>
-      </c>
-      <c r="G11" s="32" t="s">
-        <v>118</v>
-      </c>
-      <c r="H11" s="32" t="s">
+      <c r="F11" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="I11" s="32" t="s">
+      <c r="G11" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="J11" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="K11" s="35" t="n">
+      <c r="H11" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="I11" s="33" t="s">
+        <v>122</v>
+      </c>
+      <c r="J11" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="K11" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="L11" s="34" t="s">
+      <c r="L11" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M11" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N11" s="34" t="n">
+      <c r="M11" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
         <v>6</v>
       </c>
-      <c r="O11" s="37"/>
+      <c r="O11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>121</v>
-      </c>
-      <c r="B12" s="32" t="s">
-        <v>122</v>
-      </c>
-      <c r="C12" s="32" t="s">
+      <c r="A12" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="B12" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="32" t="s">
-        <v>124</v>
-      </c>
-      <c r="G12" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="H12" s="32" t="s">
+      <c r="F12" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="I12" s="32" t="s">
+      <c r="G12" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="J12" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="K12" s="35" t="n">
+      <c r="H12" s="33" t="s">
+        <v>128</v>
+      </c>
+      <c r="I12" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="J12" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="K12" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="L12" s="34" t="s">
+      <c r="L12" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M12" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N12" s="34" t="n">
+      <c r="M12" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
         <v>6</v>
       </c>
-      <c r="O12" s="37"/>
+      <c r="O12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>128</v>
-      </c>
-      <c r="B13" s="32" t="s">
-        <v>129</v>
-      </c>
-      <c r="C13" s="32" t="s">
+      <c r="A13" s="32" t="s">
         <v>130</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="B13" s="33" t="s">
+        <v>131</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="34" t="s">
+      <c r="E13" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="32" t="s">
-        <v>131</v>
-      </c>
-      <c r="G13" s="32" t="s">
-        <v>132</v>
-      </c>
-      <c r="H13" s="32" t="s">
+      <c r="F13" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="G13" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="J13" s="34" t="s">
+      <c r="H13" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="K13" s="35" t="n">
+      <c r="I13" s="33" t="s">
+        <v>136</v>
+      </c>
+      <c r="J13" s="35" t="s">
+        <v>137</v>
+      </c>
+      <c r="K13" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="L13" s="34" t="s">
+      <c r="L13" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N13" s="34" t="n">
+      <c r="M13" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
         <v>8</v>
       </c>
-      <c r="O13" s="37"/>
+      <c r="O13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>136</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>137</v>
-      </c>
-      <c r="C14" s="32" t="s">
+      <c r="A14" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="D14" s="42" t="s">
+      <c r="B14" s="33" t="s">
+        <v>139</v>
+      </c>
+      <c r="C14" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="D14" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="G14" s="32" t="s">
-        <v>140</v>
-      </c>
-      <c r="H14" s="32" t="s">
+      <c r="F14" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="G14" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="J14" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="K14" s="35" t="n">
+      <c r="H14" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="I14" s="33" t="s">
+        <v>144</v>
+      </c>
+      <c r="J14" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="K14" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="34" t="s">
+      <c r="L14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M14" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N14" s="34" t="n">
+      <c r="M14" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
         <v>4</v>
       </c>
-      <c r="O14" s="37"/>
+      <c r="O14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>143</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C15" s="32" t="s">
+      <c r="A15" s="32" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="42" t="s">
+      <c r="B15" s="33" t="s">
+        <v>146</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="D15" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="34" t="s">
+      <c r="E15" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="32" t="s">
-        <v>146</v>
-      </c>
-      <c r="G15" s="32" t="s">
-        <v>147</v>
-      </c>
-      <c r="H15" s="32" t="s">
+      <c r="F15" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="I15" s="32" t="s">
+      <c r="G15" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="J15" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="K15" s="35" t="n">
+      <c r="H15" s="33" t="s">
+        <v>150</v>
+      </c>
+      <c r="I15" s="33" t="s">
+        <v>151</v>
+      </c>
+      <c r="J15" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="K15" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L15" s="34" t="s">
+      <c r="L15" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M15" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N15" s="34" t="n">
+      <c r="M15" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
         <v>3</v>
       </c>
-      <c r="O15" s="37"/>
+      <c r="O15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>150</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>151</v>
-      </c>
-      <c r="C16" s="32" t="s">
+      <c r="A16" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="D16" s="42" t="s">
+      <c r="B16" s="33" t="s">
+        <v>153</v>
+      </c>
+      <c r="C16" s="33" t="s">
+        <v>154</v>
+      </c>
+      <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>154</v>
-      </c>
-      <c r="G16" s="32" t="s">
+      <c r="E16" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="H16" s="32" t="s">
+      <c r="F16" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="I16" s="32" t="s">
+      <c r="G16" s="33" t="s">
         <v>157</v>
       </c>
-      <c r="J16" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="K16" s="35" t="n">
+      <c r="H16" s="33" t="s">
+        <v>158</v>
+      </c>
+      <c r="I16" s="33" t="s">
+        <v>159</v>
+      </c>
+      <c r="J16" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="K16" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L16" s="34" t="s">
+      <c r="L16" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="M16" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N16" s="34" t="n">
+      <c r="M16" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
         <v>4</v>
       </c>
-      <c r="O16" s="37"/>
+      <c r="O16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="B17" s="32" t="s">
-        <v>159</v>
-      </c>
-      <c r="C17" s="32" t="s">
+      <c r="A17" s="32" t="s">
         <v>160</v>
       </c>
-      <c r="D17" s="43" t="s">
+      <c r="B17" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="C17" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="D17" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F17" s="32" t="s">
-        <v>161</v>
-      </c>
-      <c r="G17" s="32" t="s">
-        <v>162</v>
-      </c>
-      <c r="H17" s="32" t="s">
+      <c r="F17" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="G17" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="J17" s="34" t="s">
+      <c r="H17" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="K17" s="35" t="n">
+      <c r="I17" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="J17" s="35" t="s">
+        <v>167</v>
+      </c>
+      <c r="K17" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L17" s="34" t="s">
+      <c r="L17" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N17" s="34" t="n">
+      <c r="M17" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
         <v>1</v>
       </c>
-      <c r="O17" s="37"/>
+      <c r="O17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>167</v>
-      </c>
-      <c r="C18" s="32" t="s">
+      <c r="A18" s="32" t="s">
         <v>168</v>
       </c>
-      <c r="D18" s="44" t="s">
+      <c r="B18" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="C18" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="D18" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F18" s="32" t="s">
-        <v>169</v>
-      </c>
-      <c r="G18" s="32" t="s">
-        <v>170</v>
-      </c>
-      <c r="H18" s="32" t="s">
+      <c r="F18" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="G18" s="33" t="s">
         <v>172</v>
       </c>
-      <c r="J18" s="34" t="s">
+      <c r="H18" s="33" t="s">
         <v>173</v>
       </c>
-      <c r="K18" s="35" t="n">
+      <c r="I18" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="J18" s="35" t="s">
+        <v>175</v>
+      </c>
+      <c r="K18" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L18" s="34" t="s">
+      <c r="L18" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M18" s="36" t="s">
-        <v>78</v>
-      </c>
-      <c r="N18" s="34" t="n">
+      <c r="M18" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
         <v>0</v>
       </c>
-      <c r="O18" s="37"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="45" t="s">
-        <v>174</v>
-      </c>
-      <c r="B19" s="46"/>
-      <c r="C19" s="46"/>
-      <c r="D19" s="46"/>
-      <c r="E19" s="46"/>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="46"/>
-      <c r="I19" s="46"/>
-      <c r="J19" s="46"/>
-      <c r="K19" s="47" t="n">
+      <c r="O18" s="38"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="46" t="s">
+        <v>176</v>
+      </c>
+      <c r="B19" s="47"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="47"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="47"/>
+      <c r="J19" s="47"/>
+      <c r="K19" s="48" t="n">
         <f aca="false">SUM(K5:K18)</f>
         <v>27</v>
       </c>
-      <c r="L19" s="46"/>
-      <c r="M19" s="46"/>
-      <c r="N19" s="45" t="n">
+      <c r="L19" s="47"/>
+      <c r="M19" s="47"/>
+      <c r="N19" s="46" t="n">
         <f aca="false">SUM(N5:N18)</f>
         <v>49</v>
       </c>
-      <c r="O19" s="46"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K20" s="15" t="s">
-        <v>175</v>
+      <c r="O19" s="47"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K20" s="16" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:O18"/>
   <conditionalFormatting sqref="M5:M18">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:E18">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
       <formula>"Should"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L18">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M5="Done"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3530,1368 +3560,1368 @@
   <dimension ref="A1:H53"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>177</v>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
-        <v>178</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="30" t="s">
+      <c r="A4" s="31" t="s">
         <v>180</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="B4" s="31" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>182</v>
-      </c>
-      <c r="G4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>183</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="G4" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="H4" s="31" t="s">
         <v>186</v>
       </c>
-      <c r="C5" s="32" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
         <v>187</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="B5" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F5" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="G5" s="48" t="str">
+      <c r="E5" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E5,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H5" s="48" t="str">
+      <c r="H5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E5,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
+        <v>190</v>
+      </c>
+      <c r="B6" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="B6" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="34" t="s">
+      <c r="C6" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F6" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="G6" s="48" t="str">
+      <c r="E6" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E6,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H6" s="48" t="str">
+      <c r="H6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E6,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>190</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="D7" s="34" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E7" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F7" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="G7" s="48" t="str">
+      <c r="E7" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E7,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H7" s="48" t="str">
+      <c r="H7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E7,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="B8" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="C8" s="32" t="s">
-        <v>193</v>
-      </c>
-      <c r="D8" s="34" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C8" s="33" t="s">
+        <v>195</v>
+      </c>
+      <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E8" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="48" t="str">
+      <c r="E8" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="35"/>
+      <c r="G8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E8,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H8" s="48" t="str">
+      <c r="H8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E8,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>194</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>186</v>
-      </c>
-      <c r="C9" s="32" t="s">
-        <v>195</v>
-      </c>
-      <c r="D9" s="34" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
         <v>196</v>
       </c>
-      <c r="E9" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="48" t="str">
+      <c r="B9" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="C9" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="D9" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" s="35"/>
+      <c r="G9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E9,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H9" s="48" t="str">
+      <c r="H9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E9,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C10" s="32" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
         <v>199</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="B10" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="48" t="str">
+      <c r="E10" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F10" s="35"/>
+      <c r="G10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E10,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H10" s="48" t="str">
+      <c r="H10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E10,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="32" t="s">
+        <v>202</v>
+      </c>
+      <c r="B11" s="33" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>201</v>
-      </c>
-      <c r="D11" s="34" t="s">
+      <c r="C11" s="33" t="s">
+        <v>203</v>
+      </c>
+      <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E11" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="48" t="str">
+      <c r="E11" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" s="35"/>
+      <c r="G11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E11,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H11" s="48" t="str">
+      <c r="H11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E11,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>202</v>
-      </c>
-      <c r="B12" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="D12" s="34" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F12" s="34"/>
-      <c r="G12" s="48" t="str">
+      <c r="E12" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" s="35"/>
+      <c r="G12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E12,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H12" s="48" t="str">
+      <c r="H12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E12,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="B13" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>205</v>
-      </c>
-      <c r="D13" s="34" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C13" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F13" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="G13" s="48" t="str">
+      <c r="E13" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F13" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E13,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H13" s="48" t="str">
+      <c r="H13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E13,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="B14" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>207</v>
-      </c>
-      <c r="D14" s="34" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C14" s="33" t="s">
+        <v>209</v>
+      </c>
+      <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F14" s="34"/>
-      <c r="G14" s="48" t="str">
+      <c r="E14" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" s="35"/>
+      <c r="G14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E14,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H14" s="48" t="str">
+      <c r="H14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E14,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>198</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="D15" s="34" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>210</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="C15" s="33" t="s">
+        <v>211</v>
+      </c>
+      <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F15" s="34"/>
-      <c r="G15" s="48" t="str">
+      <c r="E15" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" s="35"/>
+      <c r="G15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E15,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H15" s="48" t="str">
+      <c r="H15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E15,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="B16" s="32" t="s">
-        <v>211</v>
-      </c>
-      <c r="C16" s="32" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
         <v>212</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="B16" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="C16" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="D16" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E16" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="F16" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="48" t="str">
+      <c r="E16" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E16,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H16" s="48" t="str">
+      <c r="H16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E16,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>215</v>
+      </c>
+      <c r="B17" s="33" t="s">
         <v>213</v>
       </c>
-      <c r="B17" s="32" t="s">
-        <v>211</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>214</v>
-      </c>
-      <c r="D17" s="34" t="s">
+      <c r="C17" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="D17" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="F17" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G17" s="48" t="str">
+      <c r="E17" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="F17" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H17" s="48" t="str">
+      <c r="H17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
-        <v>215</v>
-      </c>
-      <c r="B18" s="32" t="s">
-        <v>211</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>216</v>
-      </c>
-      <c r="D18" s="34" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="32" t="s">
+        <v>217</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="C18" s="33" t="s">
+        <v>218</v>
+      </c>
+      <c r="D18" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="F18" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="G18" s="48" t="str">
+      <c r="E18" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="F18" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H18" s="48" t="str">
+      <c r="H18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="B19" s="32" t="s">
-        <v>211</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>218</v>
-      </c>
-      <c r="D19" s="34" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="32" t="s">
+        <v>219</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="D19" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F19" s="34"/>
-      <c r="G19" s="48" t="str">
+      <c r="E19" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="35"/>
+      <c r="G19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E19,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H19" s="48" t="str">
+      <c r="H19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E19,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="B20" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="C20" s="32" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="32" t="s">
         <v>221</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="B20" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="D20" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F20" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G20" s="48" t="str">
+      <c r="E20" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F20" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H20" s="48" t="str">
+      <c r="H20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="31" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="B21" s="33" t="s">
         <v>222</v>
       </c>
-      <c r="B21" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>223</v>
-      </c>
-      <c r="D21" s="34" t="s">
+      <c r="C21" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="D21" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F21" s="34"/>
-      <c r="G21" s="48" t="str">
+      <c r="E21" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" s="35"/>
+      <c r="G21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E21,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H21" s="48" t="str">
+      <c r="H21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E21,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
-        <v>224</v>
-      </c>
-      <c r="B22" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="C22" s="32" t="s">
-        <v>225</v>
-      </c>
-      <c r="D22" s="34" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="B22" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="D22" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F22" s="34" t="s">
+      <c r="E22" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F22" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="G22" s="48" t="str">
+      <c r="G22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E22,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H22" s="48" t="str">
+      <c r="H22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E22,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
-        <v>226</v>
-      </c>
-      <c r="B23" s="32" t="s">
-        <v>227</v>
-      </c>
-      <c r="C23" s="32" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="32" t="s">
         <v>228</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="B23" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>230</v>
+      </c>
+      <c r="D23" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F23" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G23" s="48" t="str">
+      <c r="E23" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F23" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H23" s="48" t="str">
+      <c r="H23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="32" t="s">
+        <v>231</v>
+      </c>
+      <c r="B24" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="B24" s="32" t="s">
-        <v>227</v>
-      </c>
-      <c r="C24" s="32" t="s">
-        <v>230</v>
-      </c>
-      <c r="D24" s="34" t="s">
+      <c r="C24" s="33" t="s">
+        <v>232</v>
+      </c>
+      <c r="D24" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E24" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F24" s="34"/>
-      <c r="G24" s="48" t="str">
+      <c r="E24" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F24" s="35"/>
+      <c r="G24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E24,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H24" s="48" t="str">
+      <c r="H24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E24,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
-        <v>231</v>
-      </c>
-      <c r="B25" s="32" t="s">
-        <v>227</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>232</v>
-      </c>
-      <c r="D25" s="34" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="32" t="s">
+        <v>233</v>
+      </c>
+      <c r="B25" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="C25" s="33" t="s">
+        <v>234</v>
+      </c>
+      <c r="D25" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F25" s="34" t="s">
+      <c r="E25" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="G25" s="48" t="str">
+      <c r="G25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E25,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H25" s="48" t="str">
+      <c r="H25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E25,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
-        <v>233</v>
-      </c>
-      <c r="B26" s="32" t="s">
-        <v>234</v>
-      </c>
-      <c r="C26" s="32" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="32" t="s">
         <v>235</v>
       </c>
-      <c r="D26" s="34" t="s">
+      <c r="B26" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>237</v>
+      </c>
+      <c r="D26" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F26" s="34"/>
-      <c r="G26" s="48" t="str">
+      <c r="E26" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F26" s="35"/>
+      <c r="G26" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E26,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H26" s="48" t="str">
+      <c r="H26" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E26,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="32" t="s">
+        <v>238</v>
+      </c>
+      <c r="B27" s="33" t="s">
         <v>236</v>
       </c>
-      <c r="B27" s="32" t="s">
-        <v>234</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>237</v>
-      </c>
-      <c r="D27" s="34" t="s">
+      <c r="C27" s="33" t="s">
+        <v>239</v>
+      </c>
+      <c r="D27" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F27" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="G27" s="48" t="str">
+      <c r="E27" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F27" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H27" s="48" t="str">
+      <c r="H27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="31" t="s">
-        <v>238</v>
-      </c>
-      <c r="B28" s="32" t="s">
-        <v>234</v>
-      </c>
-      <c r="C28" s="32" t="s">
-        <v>239</v>
-      </c>
-      <c r="D28" s="34" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="B28" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>241</v>
+      </c>
+      <c r="D28" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F28" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="G28" s="48" t="str">
+      <c r="E28" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F28" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E28,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H28" s="48" t="str">
+      <c r="H28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E28,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31" t="s">
-        <v>240</v>
-      </c>
-      <c r="B29" s="32" t="s">
-        <v>234</v>
-      </c>
-      <c r="C29" s="32" t="s">
-        <v>241</v>
-      </c>
-      <c r="D29" s="34" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="B29" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F29" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="G29" s="48" t="str">
+      <c r="E29" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F29" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E29,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H29" s="48" t="str">
+      <c r="H29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E29,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="31" t="s">
-        <v>242</v>
-      </c>
-      <c r="B30" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C30" s="32" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
         <v>244</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="B30" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>246</v>
+      </c>
+      <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F30" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="G30" s="48" t="str">
+      <c r="E30" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="F30" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="G30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E30,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H30" s="48" t="str">
+      <c r="H30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E30,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="B31" s="33" t="s">
         <v>245</v>
       </c>
-      <c r="B31" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C31" s="32" t="s">
-        <v>246</v>
-      </c>
-      <c r="D31" s="34" t="s">
+      <c r="C31" s="33" t="s">
+        <v>248</v>
+      </c>
+      <c r="D31" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F31" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="G31" s="48" t="str">
+      <c r="E31" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="F31" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H31" s="48" t="str">
+      <c r="H31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="31" t="s">
-        <v>247</v>
-      </c>
-      <c r="B32" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C32" s="32" t="s">
-        <v>248</v>
-      </c>
-      <c r="D32" s="34" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="C32" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E32" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F32" s="34"/>
-      <c r="G32" s="48" t="str">
+      <c r="E32" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="F32" s="35"/>
+      <c r="G32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E32,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H32" s="48" t="str">
+      <c r="H32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E32,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="B33" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C33" s="32" t="s">
-        <v>250</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="E33" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F33" s="34"/>
-      <c r="G33" s="48" t="str">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="32" t="s">
+        <v>251</v>
+      </c>
+      <c r="B33" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>252</v>
+      </c>
+      <c r="D33" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E33" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="F33" s="35"/>
+      <c r="G33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E33,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H33" s="48" t="str">
+      <c r="H33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E33,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31" t="s">
-        <v>251</v>
-      </c>
-      <c r="B34" s="32" t="s">
-        <v>243</v>
-      </c>
-      <c r="C34" s="32" t="s">
-        <v>252</v>
-      </c>
-      <c r="D34" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="E34" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F34" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="G34" s="48" t="str">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="32" t="s">
+        <v>253</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="C34" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="D34" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="F34" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="G34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E34,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H34" s="48" t="str">
+      <c r="H34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E34,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="31" t="s">
-        <v>253</v>
-      </c>
-      <c r="B35" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="C35" s="32" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D35" s="34" t="s">
+      <c r="B35" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="C35" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E35" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="F35" s="34"/>
-      <c r="G35" s="48" t="str">
+      <c r="E35" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="F35" s="35"/>
+      <c r="G35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E35,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H35" s="48" t="str">
+      <c r="H35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E35,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="31" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="B36" s="33" t="s">
         <v>256</v>
       </c>
-      <c r="B36" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="C36" s="32" t="s">
-        <v>257</v>
-      </c>
-      <c r="D36" s="34" t="s">
+      <c r="C36" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E36" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="F36" s="34"/>
-      <c r="G36" s="48" t="str">
+      <c r="E36" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="F36" s="35"/>
+      <c r="G36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E36,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H36" s="48" t="str">
+      <c r="H36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E36,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="B37" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="C37" s="32" t="s">
-        <v>259</v>
-      </c>
-      <c r="D37" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="E37" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="F37" s="34"/>
-      <c r="G37" s="48" t="str">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="C37" s="33" t="s">
+        <v>261</v>
+      </c>
+      <c r="D37" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="E37" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="F37" s="35"/>
+      <c r="G37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E37,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H37" s="48" t="str">
+      <c r="H37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E37,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="31" t="s">
-        <v>260</v>
-      </c>
-      <c r="B38" s="32" t="s">
-        <v>261</v>
-      </c>
-      <c r="C38" s="32" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32" t="s">
         <v>262</v>
       </c>
-      <c r="D38" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="E38" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="F38" s="34"/>
-      <c r="G38" s="48" t="str">
+      <c r="B38" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="C38" s="33" t="s">
+        <v>264</v>
+      </c>
+      <c r="D38" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="E38" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F38" s="35"/>
+      <c r="G38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E38,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H38" s="48" t="str">
+      <c r="H38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E38,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="31" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="B39" s="33" t="s">
         <v>263</v>
       </c>
-      <c r="B39" s="32" t="s">
-        <v>261</v>
-      </c>
-      <c r="C39" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="D39" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="E39" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="F39" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="G39" s="48" t="str">
+      <c r="C39" s="33" t="s">
+        <v>266</v>
+      </c>
+      <c r="D39" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="E39" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F39" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="G39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E39,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H39" s="48" t="str">
+      <c r="H39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E39,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="B40" s="32" t="s">
-        <v>261</v>
-      </c>
-      <c r="C40" s="32" t="s">
-        <v>266</v>
-      </c>
-      <c r="D40" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="E40" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="F40" s="34"/>
-      <c r="G40" s="48" t="str">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="C40" s="33" t="s">
+        <v>268</v>
+      </c>
+      <c r="D40" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F40" s="35"/>
+      <c r="G40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E40,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H40" s="48" t="str">
+      <c r="H40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E40,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="31" t="s">
-        <v>267</v>
-      </c>
-      <c r="B41" s="32" t="s">
-        <v>268</v>
-      </c>
-      <c r="C41" s="32" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="32" t="s">
         <v>269</v>
       </c>
-      <c r="D41" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="E41" s="34" t="s">
-        <v>150</v>
-      </c>
-      <c r="F41" s="34"/>
-      <c r="G41" s="48" t="str">
+      <c r="B41" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C41" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="D41" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="E41" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="F41" s="35"/>
+      <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E41,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H41" s="48" t="str">
+      <c r="H41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E41,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="31" t="s">
-        <v>270</v>
-      </c>
-      <c r="B42" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C42" s="32" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="32" t="s">
         <v>272</v>
       </c>
-      <c r="D42" s="34" t="s">
+      <c r="B42" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="C42" s="33" t="s">
+        <v>274</v>
+      </c>
+      <c r="D42" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F42" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="G42" s="48" t="str">
+      <c r="E42" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F42" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H42" s="48" t="str">
+      <c r="H42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="31" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="B43" s="33" t="s">
         <v>273</v>
       </c>
-      <c r="B43" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C43" s="32" t="s">
-        <v>274</v>
-      </c>
-      <c r="D43" s="34" t="s">
+      <c r="C43" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="D43" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E43" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F43" s="34"/>
-      <c r="G43" s="48" t="str">
+      <c r="E43" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F43" s="35"/>
+      <c r="G43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E43,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H43" s="48" t="str">
+      <c r="H43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E43,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="31" t="s">
-        <v>275</v>
-      </c>
-      <c r="B44" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C44" s="32" t="s">
-        <v>276</v>
-      </c>
-      <c r="D44" s="34" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="B44" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="C44" s="33" t="s">
+        <v>278</v>
+      </c>
+      <c r="D44" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F44" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="G44" s="48" t="str">
+      <c r="E44" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F44" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H44" s="48" t="str">
+      <c r="H44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="31" t="s">
-        <v>277</v>
-      </c>
-      <c r="B45" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C45" s="32" t="s">
-        <v>278</v>
-      </c>
-      <c r="D45" s="34" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="B45" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>280</v>
+      </c>
+      <c r="D45" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E45" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F45" s="34"/>
-      <c r="G45" s="48" t="str">
+      <c r="E45" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F45" s="35"/>
+      <c r="G45" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E45,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H45" s="48" t="str">
+      <c r="H45" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E45,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="31" t="s">
-        <v>279</v>
-      </c>
-      <c r="B46" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C46" s="32" t="s">
-        <v>280</v>
-      </c>
-      <c r="D46" s="34" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="C46" s="33" t="s">
+        <v>282</v>
+      </c>
+      <c r="D46" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E46" s="34" t="s">
-        <v>93</v>
-      </c>
-      <c r="F46" s="34"/>
-      <c r="G46" s="48" t="str">
+      <c r="E46" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="F46" s="35"/>
+      <c r="G46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E46,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H46" s="48" t="str">
+      <c r="H46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E46,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="31" t="s">
-        <v>281</v>
-      </c>
-      <c r="B47" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C47" s="32" t="s">
-        <v>282</v>
-      </c>
-      <c r="D47" s="34" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="B47" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="C47" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="F47" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="G47" s="48" t="str">
+      <c r="E47" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H47" s="48" t="str">
+      <c r="H47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="31" t="s">
-        <v>283</v>
-      </c>
-      <c r="B48" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C48" s="32" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="32" t="s">
         <v>285</v>
       </c>
-      <c r="D48" s="34" t="s">
+      <c r="B48" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C48" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E48" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F48" s="34" t="s">
+      <c r="E48" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="F48" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="G48" s="48" t="str">
+      <c r="G48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E48,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H48" s="48" t="str">
+      <c r="H48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E48,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="31" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="32" t="s">
+        <v>288</v>
+      </c>
+      <c r="B49" s="33" t="s">
         <v>286</v>
       </c>
-      <c r="B49" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C49" s="32" t="s">
-        <v>287</v>
-      </c>
-      <c r="D49" s="34" t="s">
+      <c r="C49" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="D49" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E49" s="34" t="s">
+      <c r="E49" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="F49" s="34"/>
-      <c r="G49" s="48" t="str">
+      <c r="F49" s="35"/>
+      <c r="G49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E49,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H49" s="48" t="str">
+      <c r="H49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E49,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="31" t="s">
-        <v>288</v>
-      </c>
-      <c r="B50" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C50" s="32" t="s">
-        <v>289</v>
-      </c>
-      <c r="D50" s="34" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="32" t="s">
+        <v>290</v>
+      </c>
+      <c r="B50" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C50" s="33" t="s">
+        <v>291</v>
+      </c>
+      <c r="D50" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="34" t="s">
-        <v>114</v>
-      </c>
-      <c r="F50" s="34"/>
-      <c r="G50" s="48" t="str">
+      <c r="E50" s="35" t="s">
+        <v>116</v>
+      </c>
+      <c r="F50" s="35"/>
+      <c r="G50" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E50,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H50" s="48" t="str">
+      <c r="H50" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E50,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="31" t="s">
-        <v>290</v>
-      </c>
-      <c r="B51" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C51" s="32" t="s">
-        <v>291</v>
-      </c>
-      <c r="D51" s="34" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="32" t="s">
+        <v>292</v>
+      </c>
+      <c r="B51" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C51" s="33" t="s">
+        <v>293</v>
+      </c>
+      <c r="D51" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F51" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="G51" s="48" t="str">
+      <c r="E51" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F51" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H51" s="48" t="str">
+      <c r="H51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="31" t="s">
-        <v>292</v>
-      </c>
-      <c r="B52" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C52" s="32" t="s">
-        <v>293</v>
-      </c>
-      <c r="D52" s="34" t="s">
-        <v>153</v>
-      </c>
-      <c r="E52" s="34" t="s">
-        <v>107</v>
-      </c>
-      <c r="F52" s="34"/>
-      <c r="G52" s="48" t="str">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="32" t="s">
+        <v>294</v>
+      </c>
+      <c r="B52" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C52" s="33" t="s">
+        <v>295</v>
+      </c>
+      <c r="D52" s="35" t="s">
+        <v>155</v>
+      </c>
+      <c r="E52" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F52" s="35"/>
+      <c r="G52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E52,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H52" s="48" t="str">
+      <c r="H52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E52,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="s">
-        <v>294</v>
-      </c>
-      <c r="B53" s="32" t="s">
-        <v>284</v>
-      </c>
-      <c r="C53" s="32" t="s">
-        <v>295</v>
-      </c>
-      <c r="D53" s="34" t="s">
-        <v>196</v>
-      </c>
-      <c r="E53" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="F53" s="34"/>
-      <c r="G53" s="48" t="str">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="32" t="s">
+        <v>296</v>
+      </c>
+      <c r="B53" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="C53" s="33" t="s">
+        <v>297</v>
+      </c>
+      <c r="D53" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E53" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="F53" s="35"/>
+      <c r="G53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E53,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H53" s="48" t="str">
+      <c r="H53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E53,'PR Plan'!$A$5:$A$18,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
@@ -4899,21 +4929,21 @@
   </sheetData>
   <autoFilter ref="A4:H53"/>
   <conditionalFormatting sqref="G5:G53">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D53">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Must"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4936,321 +4966,321 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>297</v>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
-        <v>298</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>299</v>
-      </c>
-      <c r="C4" s="30" t="s">
+      <c r="A4" s="31" t="s">
         <v>300</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>301</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>302</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>303</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>304</v>
       </c>
+      <c r="F4" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
-        <v>305</v>
-      </c>
-      <c r="B5" s="34" t="s">
-        <v>306</v>
-      </c>
-      <c r="C5" s="49" t="s">
+      <c r="A5" s="32" t="s">
         <v>307</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="B5" s="35" t="s">
         <v>308</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="C5" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="D5" s="33" t="s">
         <v>310</v>
       </c>
-      <c r="G5" s="34" t="s">
-        <v>114</v>
+      <c r="E5" s="33" t="s">
+        <v>311</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="35" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>311</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>312</v>
-      </c>
-      <c r="C6" s="49" t="s">
+      <c r="A6" s="32" t="s">
         <v>313</v>
       </c>
-      <c r="D6" s="32" t="s">
+      <c r="B6" s="35" t="s">
         <v>314</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="C6" s="50" t="s">
         <v>315</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="D6" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="G6" s="34" t="s">
-        <v>107</v>
+      <c r="E6" s="33" t="s">
+        <v>317</v>
+      </c>
+      <c r="F6" s="33" t="s">
+        <v>318</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>317</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>318</v>
-      </c>
-      <c r="C7" s="49" t="s">
+      <c r="A7" s="32" t="s">
         <v>319</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="B7" s="35" t="s">
         <v>320</v>
       </c>
-      <c r="E7" s="32" t="s">
+      <c r="C7" s="50" t="s">
         <v>321</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="D7" s="33" t="s">
         <v>322</v>
       </c>
-      <c r="G7" s="34" t="s">
-        <v>100</v>
+      <c r="E7" s="33" t="s">
+        <v>323</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>324</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>323</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>324</v>
-      </c>
-      <c r="C8" s="49" t="s">
+      <c r="A8" s="32" t="s">
         <v>325</v>
       </c>
-      <c r="D8" s="32" t="s">
+      <c r="B8" s="35" t="s">
         <v>326</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="C8" s="50" t="s">
         <v>327</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="D8" s="33" t="s">
         <v>328</v>
       </c>
-      <c r="G8" s="34" t="s">
-        <v>93</v>
+      <c r="E8" s="33" t="s">
+        <v>329</v>
+      </c>
+      <c r="F8" s="33" t="s">
+        <v>330</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>329</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>330</v>
-      </c>
-      <c r="C9" s="49" t="s">
+      <c r="A9" s="32" t="s">
         <v>331</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="B9" s="35" t="s">
         <v>332</v>
       </c>
-      <c r="E9" s="32" t="s">
+      <c r="C9" s="50" t="s">
         <v>333</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="D9" s="33" t="s">
         <v>334</v>
       </c>
-      <c r="G9" s="34" t="s">
+      <c r="E9" s="33" t="s">
+        <v>335</v>
+      </c>
+      <c r="F9" s="33" t="s">
+        <v>336</v>
+      </c>
+      <c r="G9" s="35" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>335</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="C10" s="49" t="s">
+      <c r="A10" s="32" t="s">
         <v>337</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="B10" s="35" t="s">
         <v>338</v>
       </c>
-      <c r="E10" s="32" t="s">
+      <c r="C10" s="50" t="s">
         <v>339</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="D10" s="33" t="s">
         <v>340</v>
       </c>
-      <c r="G10" s="34" t="s">
-        <v>114</v>
+      <c r="E10" s="33" t="s">
+        <v>341</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>342</v>
+      </c>
+      <c r="G10" s="35" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
-        <v>341</v>
-      </c>
-      <c r="B11" s="34" t="s">
+      <c r="A11" s="32" t="s">
+        <v>343</v>
+      </c>
+      <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="49" t="s">
-        <v>342</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>343</v>
-      </c>
-      <c r="E11" s="32" t="s">
+      <c r="C11" s="50" t="s">
         <v>344</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="D11" s="33" t="s">
         <v>345</v>
       </c>
-      <c r="G11" s="34" t="s">
-        <v>128</v>
+      <c r="E11" s="33" t="s">
+        <v>346</v>
+      </c>
+      <c r="F11" s="33" t="s">
+        <v>347</v>
+      </c>
+      <c r="G11" s="35" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>346</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>347</v>
-      </c>
-      <c r="C12" s="49" t="s">
+      <c r="A12" s="32" t="s">
         <v>348</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="B12" s="35" t="s">
         <v>349</v>
       </c>
-      <c r="E12" s="32" t="s">
+      <c r="C12" s="50" t="s">
         <v>350</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="D12" s="33" t="s">
         <v>351</v>
       </c>
-      <c r="G12" s="34" t="s">
-        <v>107</v>
+      <c r="E12" s="33" t="s">
+        <v>352</v>
+      </c>
+      <c r="F12" s="33" t="s">
+        <v>353</v>
+      </c>
+      <c r="G12" s="35" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>352</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>353</v>
-      </c>
-      <c r="C13" s="49" t="s">
+      <c r="A13" s="32" t="s">
         <v>354</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="B13" s="35" t="s">
         <v>355</v>
       </c>
-      <c r="E13" s="32" t="s">
+      <c r="C13" s="50" t="s">
         <v>356</v>
       </c>
-      <c r="F13" s="32" t="s">
+      <c r="D13" s="33" t="s">
         <v>357</v>
       </c>
-      <c r="G13" s="34" t="s">
-        <v>107</v>
+      <c r="E13" s="33" t="s">
+        <v>358</v>
+      </c>
+      <c r="F13" s="33" t="s">
+        <v>359</v>
+      </c>
+      <c r="G13" s="35" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>358</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>359</v>
-      </c>
-      <c r="C14" s="49" t="s">
+      <c r="A14" s="32" t="s">
         <v>360</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="B14" s="35" t="s">
         <v>361</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="C14" s="50" t="s">
         <v>362</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="D14" s="33" t="s">
         <v>363</v>
       </c>
-      <c r="G14" s="34" t="s">
+      <c r="E14" s="33" t="s">
+        <v>364</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>365</v>
+      </c>
+      <c r="G14" s="35" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>364</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>365</v>
-      </c>
-      <c r="C15" s="49" t="s">
+      <c r="A15" s="32" t="s">
         <v>366</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="B15" s="35" t="s">
         <v>367</v>
       </c>
-      <c r="E15" s="32" t="s">
+      <c r="C15" s="50" t="s">
         <v>368</v>
       </c>
-      <c r="F15" s="32" t="s">
+      <c r="D15" s="33" t="s">
         <v>369</v>
       </c>
-      <c r="G15" s="34" t="s">
+      <c r="E15" s="33" t="s">
+        <v>370</v>
+      </c>
+      <c r="F15" s="33" t="s">
+        <v>371</v>
+      </c>
+      <c r="G15" s="35" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>370</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>371</v>
-      </c>
-      <c r="C16" s="49" t="s">
+      <c r="A16" s="32" t="s">
         <v>372</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="B16" s="35" t="s">
         <v>373</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="C16" s="50" t="s">
         <v>374</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="D16" s="33" t="s">
         <v>375</v>
       </c>
-      <c r="G16" s="34" t="s">
+      <c r="E16" s="33" t="s">
+        <v>376</v>
+      </c>
+      <c r="F16" s="33" t="s">
+        <v>377</v>
+      </c>
+      <c r="G16" s="35" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark PR-02 done in the delivery plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -323,10 +323,7 @@
     <t xml:space="preserve">Invariants in the schema not the app; why tool_calls separate from messages; HNSW vs IVFFlat; denormalised business_id on chunks; one conversation per session</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design doc reviewed and merged first (PR #2, docs/database-design.md)</t>
+    <t xml:space="preserve">Merged: PR #3. Design doc reviewed first (PR #2). Three review rounds; verified as service_role.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-03</t>
@@ -352,6 +349,9 @@
   </si>
   <si>
     <t xml:space="preserve">Why test data is designed around the demo questions; why include a PDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-04</t>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.0185185185185185</v>
+        <v>0.0740740740740741</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="D27" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A27,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2906,25 +2906,25 @@
         <v>19</v>
       </c>
       <c r="M6" s="37" t="s">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="N6" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A6)</f>
         <v>1</v>
       </c>
       <c r="O6" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="C7" s="33" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>90</v>
       </c>
       <c r="D7" s="34" t="s">
         <v>30</v>
@@ -2933,16 +2933,16 @@
         <v>72</v>
       </c>
       <c r="F7" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="H7" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="H7" s="33" t="s">
+      <c r="I7" s="33" t="s">
         <v>93</v>
-      </c>
-      <c r="I7" s="33" t="s">
-        <v>94</v>
       </c>
       <c r="J7" s="35" t="s">
         <v>79</v>
@@ -2954,7 +2954,7 @@
         <v>19</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N7" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A7)</f>
@@ -3000,7 +3000,7 @@
         <v>19</v>
       </c>
       <c r="M8" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N8" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A8)</f>
@@ -3046,7 +3046,7 @@
         <v>19</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
@@ -3092,7 +3092,7 @@
         <v>19</v>
       </c>
       <c r="M10" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
@@ -3138,7 +3138,7 @@
         <v>20</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
@@ -3184,7 +3184,7 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
@@ -3230,7 +3230,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3276,7 +3276,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3322,7 +3322,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3368,7 +3368,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3414,7 +3414,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3460,7 +3460,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -4813,7 +4813,7 @@
       <c r="F49" s="35"/>
       <c r="G49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E49,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E49,'PR Plan'!$A$5:$A$18,0)),"-")</f>

</xml_diff>

<commit_message>
Mark PR-03 done in the delivery plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="379">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -351,7 +351,7 @@
     <t xml:space="preserve">Why test data is designed around the demo questions; why include a PDF</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #4. Data lives in data/sample-clinic/ (not docs/). PDF export needed the Writer filter.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-04</t>
@@ -382,6 +382,9 @@
   </si>
   <si>
     <t xml:space="preserve">Chunk size &amp; overlap reasoning; heading prefix (contextual chunks); why tokens not words; embedding model choice &amp; cost; idempotent ingestion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-05</t>
@@ -2303,7 +2306,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2339,7 +2342,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2348,7 +2351,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.0740740740740741</v>
+        <v>0.0925925925925926</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2539,7 +2542,7 @@
       </c>
       <c r="D27" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A27,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2954,13 +2957,15 @@
         <v>19</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="N7" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A7)</f>
         <v>0</v>
       </c>
-      <c r="O7" s="38"/>
+      <c r="O7" s="38" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
@@ -3000,7 +3005,7 @@
         <v>19</v>
       </c>
       <c r="M8" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N8" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A8)</f>
@@ -3010,13 +3015,13 @@
     </row>
     <row r="9" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" s="39" t="s">
         <v>31</v>
@@ -3025,16 +3030,16 @@
         <v>72</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G9" s="33" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H9" s="33" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I9" s="33" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J9" s="35" t="s">
         <v>95</v>
@@ -3046,7 +3051,7 @@
         <v>19</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
@@ -3056,13 +3061,13 @@
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D10" s="40" t="s">
         <v>32</v>
@@ -3071,19 +3076,19 @@
         <v>72</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H10" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I10" s="33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J10" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K10" s="36" t="n">
         <v>2.5</v>
@@ -3092,7 +3097,7 @@
         <v>19</v>
       </c>
       <c r="M10" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
@@ -3102,13 +3107,13 @@
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D11" s="40" t="s">
         <v>32</v>
@@ -3117,19 +3122,19 @@
         <v>72</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I11" s="33" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J11" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K11" s="36" t="n">
         <v>2.5</v>
@@ -3138,7 +3143,7 @@
         <v>20</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
@@ -3148,13 +3153,13 @@
     </row>
     <row r="12" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>33</v>
@@ -3163,19 +3168,19 @@
         <v>72</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J12" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K12" s="36" t="n">
         <v>3</v>
@@ -3184,7 +3189,7 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
@@ -3194,13 +3199,13 @@
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>34</v>
@@ -3209,19 +3214,19 @@
         <v>72</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J13" s="35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K13" s="36" t="n">
         <v>4</v>
@@ -3230,7 +3235,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3240,13 +3245,13 @@
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>35</v>
@@ -3255,16 +3260,16 @@
         <v>72</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J14" s="35" t="s">
         <v>95</v>
@@ -3276,7 +3281,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3286,13 +3291,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3301,19 +3306,19 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J15" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K15" s="36" t="n">
         <v>1.5</v>
@@ -3322,7 +3327,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3332,34 +3337,34 @@
     </row>
     <row r="16" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J16" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K16" s="36" t="n">
         <v>2</v>
@@ -3368,7 +3373,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3378,13 +3383,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3393,19 +3398,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3414,7 +3419,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3424,13 +3429,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3439,19 +3444,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3460,7 +3465,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3470,7 +3475,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B19" s="47"/>
       <c r="C19" s="47"/>
@@ -3495,7 +3500,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K20" s="16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -3572,58 +3577,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E5,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3636,22 +3641,22 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E6,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3664,22 +3669,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E7,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3692,19 +3697,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
@@ -3718,19 +3723,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
@@ -3744,19 +3749,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
@@ -3770,19 +3775,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
@@ -3796,19 +3801,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
@@ -3822,22 +3827,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E13,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3850,19 +3855,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
@@ -3876,19 +3881,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
@@ -3902,19 +3907,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F16" s="35" t="s">
         <v>95</v>
@@ -3930,22 +3935,22 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E17" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3958,22 +3963,22 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3986,19 +3991,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F19" s="35"/>
       <c r="G19" s="49" t="str">
@@ -4012,22 +4017,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4040,19 +4045,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F21" s="35"/>
       <c r="G21" s="49" t="str">
@@ -4066,19 +4071,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F22" s="35" t="s">
         <v>79</v>
@@ -4094,22 +4099,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F23" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4122,19 +4127,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F24" s="35"/>
       <c r="G24" s="49" t="str">
@@ -4148,19 +4153,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F25" s="35" t="s">
         <v>79</v>
@@ -4176,19 +4181,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F26" s="35"/>
       <c r="G26" s="49" t="str">
@@ -4202,22 +4207,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F27" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4230,22 +4235,22 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F28" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E28,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4258,22 +4263,22 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E29,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4286,19 +4291,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>95</v>
@@ -4314,13 +4319,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4329,7 +4334,7 @@
         <v>95</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4342,19 +4347,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
@@ -4368,19 +4373,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
@@ -4394,22 +4399,22 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F34" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E34,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4422,19 +4427,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4448,19 +4453,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4474,19 +4479,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4500,19 +4505,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4526,22 +4531,22 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F39" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E39,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4554,19 +4559,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4580,19 +4585,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F41" s="35"/>
       <c r="G41" s="49" t="str">
@@ -4606,22 +4611,22 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4634,19 +4639,19 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E43" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F43" s="35"/>
       <c r="G43" s="49" t="str">
@@ -4660,22 +4665,22 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4688,19 +4693,19 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F45" s="35"/>
       <c r="G45" s="49" t="str">
@@ -4714,13 +4719,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4740,22 +4745,22 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4768,19 +4773,19 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E48" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F48" s="35" t="s">
         <v>69</v>
@@ -4796,13 +4801,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4822,19 +4827,19 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E50" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F50" s="35"/>
       <c r="G50" s="49" t="str">
@@ -4848,22 +4853,22 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E51" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4876,19 +4881,19 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E52" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F52" s="35"/>
       <c r="G52" s="49" t="str">
@@ -4902,19 +4907,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -4977,124 +4982,124 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G7" s="35" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5102,22 +5107,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5125,114 +5130,114 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5240,22 +5245,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5263,22 +5268,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Mark PR-04 done in the delivery plan
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="380">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -384,7 +384,7 @@
     <t xml:space="preserve">Chunk size &amp; overlap reasoning; heading prefix (contextual chunks); why tokens not words; embedding model choice &amp; cost; idempotent ingestion</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #5. Verified with real embeddings (60 chunks). Finding for PR-05: a single similarity threshold can't separate found/not-found.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-05</t>
@@ -411,6 +411,9 @@
   </si>
   <si>
     <t xml:space="preserve">Top-k choice; how the threshold was picked (eval, not guess); why sources come from retrieval not the LLM; hybrid search as next step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-06</t>
@@ -2306,7 +2309,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2342,7 +2345,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2351,7 +2354,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.0925925925925926</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2369,7 +2372,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2559,7 +2562,7 @@
       </c>
       <c r="D28" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A28,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3005,13 +3008,15 @@
         <v>19</v>
       </c>
       <c r="M8" s="37" t="s">
-        <v>102</v>
+        <v>29</v>
       </c>
       <c r="N8" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A8)</f>
         <v>2</v>
       </c>
-      <c r="O8" s="38"/>
+      <c r="O8" s="38" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
@@ -3051,7 +3056,7 @@
         <v>19</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
@@ -3061,13 +3066,13 @@
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D10" s="40" t="s">
         <v>32</v>
@@ -3076,16 +3081,16 @@
         <v>72</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G10" s="33" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H10" s="33" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I10" s="33" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J10" s="35" t="s">
         <v>103</v>
@@ -3097,7 +3102,7 @@
         <v>19</v>
       </c>
       <c r="M10" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
@@ -3107,13 +3112,13 @@
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D11" s="40" t="s">
         <v>32</v>
@@ -3122,19 +3127,19 @@
         <v>72</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I11" s="33" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J11" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K11" s="36" t="n">
         <v>2.5</v>
@@ -3143,7 +3148,7 @@
         <v>20</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
@@ -3153,13 +3158,13 @@
     </row>
     <row r="12" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>33</v>
@@ -3168,19 +3173,19 @@
         <v>72</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J12" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K12" s="36" t="n">
         <v>3</v>
@@ -3189,7 +3194,7 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
@@ -3199,13 +3204,13 @@
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>34</v>
@@ -3214,19 +3219,19 @@
         <v>72</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J13" s="35" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K13" s="36" t="n">
         <v>4</v>
@@ -3235,7 +3240,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3245,13 +3250,13 @@
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>35</v>
@@ -3260,16 +3265,16 @@
         <v>72</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J14" s="35" t="s">
         <v>95</v>
@@ -3281,7 +3286,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3291,13 +3296,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3306,19 +3311,19 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J15" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K15" s="36" t="n">
         <v>1.5</v>
@@ -3327,7 +3332,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3337,34 +3342,34 @@
     </row>
     <row r="16" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="J16" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K16" s="36" t="n">
         <v>2</v>
@@ -3373,7 +3378,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3383,13 +3388,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3398,19 +3403,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3419,7 +3424,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3429,13 +3434,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3444,19 +3449,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3465,7 +3470,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3475,7 +3480,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B19" s="47"/>
       <c r="C19" s="47"/>
@@ -3500,7 +3505,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K20" s="16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -3577,58 +3582,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E5,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3641,22 +3646,22 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E6,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3669,22 +3674,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E7,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3697,19 +3702,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
@@ -3723,19 +3728,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
@@ -3749,19 +3754,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
@@ -3775,19 +3780,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
@@ -3801,19 +3806,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
@@ -3827,22 +3832,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F13" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E13,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3855,19 +3860,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
@@ -3881,19 +3886,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
@@ -3907,13 +3912,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -3935,13 +3940,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -3950,7 +3955,7 @@
         <v>103</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3963,13 +3968,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -3978,7 +3983,7 @@
         <v>103</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3991,19 +3996,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F19" s="35"/>
       <c r="G19" s="49" t="str">
@@ -4017,22 +4022,22 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4045,19 +4050,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E21" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F21" s="35"/>
       <c r="G21" s="49" t="str">
@@ -4071,19 +4076,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F22" s="35" t="s">
         <v>79</v>
@@ -4099,22 +4104,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E23" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F23" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4127,19 +4132,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E24" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F24" s="35"/>
       <c r="G24" s="49" t="str">
@@ -4153,19 +4158,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E25" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F25" s="35" t="s">
         <v>79</v>
@@ -4181,19 +4186,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F26" s="35"/>
       <c r="G26" s="49" t="str">
@@ -4207,22 +4212,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F27" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4235,22 +4240,22 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F28" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E28,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4263,22 +4268,22 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E29,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4291,19 +4296,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>95</v>
@@ -4319,13 +4324,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4334,11 +4339,11 @@
         <v>95</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4347,19 +4352,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
@@ -4373,19 +4378,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
@@ -4399,19 +4404,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F34" s="35" t="s">
         <v>103</v>
@@ -4427,19 +4432,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4453,19 +4458,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4479,19 +4484,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4505,19 +4510,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4531,22 +4536,22 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F39" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E39,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4559,19 +4564,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4585,19 +4590,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F41" s="35"/>
       <c r="G41" s="49" t="str">
@@ -4611,22 +4616,22 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E42" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4639,19 +4644,19 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E43" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F43" s="35"/>
       <c r="G43" s="49" t="str">
@@ -4665,22 +4670,22 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4693,19 +4698,19 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F45" s="35"/>
       <c r="G45" s="49" t="str">
@@ -4719,13 +4724,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4736,7 +4741,7 @@
       <c r="F46" s="35"/>
       <c r="G46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E46,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E46,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4745,22 +4750,22 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4773,19 +4778,19 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E48" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F48" s="35" t="s">
         <v>69</v>
@@ -4801,13 +4806,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4827,19 +4832,19 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E50" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F50" s="35"/>
       <c r="G50" s="49" t="str">
@@ -4853,22 +4858,22 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E51" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4881,19 +4886,19 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E52" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F52" s="35"/>
       <c r="G52" s="49" t="str">
@@ -4907,19 +4912,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -4982,101 +4987,101 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G6" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5084,22 +5089,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5107,22 +5112,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5130,114 +5135,114 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G12" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G13" s="35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5245,22 +5250,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5268,22 +5273,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Record the hybrid-retrieval decision in the plan (D-03, D-13)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="386">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -400,7 +400,7 @@
   </si>
   <si>
     <t xml:space="preserve">- retrieve(businessId, query): embed query -&gt; match_chunks top 6
-- Similarity threshold -&gt; {found:false} when nothing relevant
+- Hybrid search (vector + full-text, RRF) and a found rule -&gt; {found:false} when nothing relevant
 - Return sources: documentId, title, heading, excerpt, similarity
 - Eval script: ~10 demo questions + expected source doc, prints hit/miss</t>
   </si>
@@ -410,7 +410,7 @@
 - Threshold value documented with the reasoning</t>
   </si>
   <si>
-    <t xml:space="preserve">Top-k choice; how the threshold was picked (eval, not guess); why sources come from retrieval not the LLM; hybrid search as next step</t>
+    <t xml:space="preserve">Why hybrid instead of a similarity threshold (measured: 0.27 correct vs 0.42 wrong); RRF; what a 'topic keyword' is and why frame verbs are excluded; sources come from retrieval not the LLM; reranker as the production next step</t>
   </si>
   <si>
     <t xml:space="preserve">Not started</t>
@@ -1113,7 +1113,7 @@
     <t xml:space="preserve">Hallucination</t>
   </si>
   <si>
-    <t xml:space="preserve">Layered: grounding prompt + similarity threshold + sources from retrieval + no facts in prompt</t>
+    <t xml:space="preserve">Layered: grounding prompt + hybrid retrieval found-rule + sources only from retrieval + no facts in prompt</t>
   </si>
   <si>
     <t xml:space="preserve">Prompt-only 'don't make things up'</t>
@@ -1122,7 +1122,7 @@
     <t xml:space="preserve">Each layer catches what the previous misses; citations cannot be invented</t>
   </si>
   <si>
-    <t xml:space="preserve">Threshold too high -&gt; false 'I don't know'; tuned with eval script</t>
+    <t xml:space="preserve">Originally planned a similarity threshold as layer 2; measurement showed it cannot work (see D-13). The retrieval gate filters noise; the prompt is the main defence</t>
   </si>
   <si>
     <t xml:space="preserve">D-04</t>
@@ -1282,6 +1282,24 @@
   </si>
   <si>
     <t xml:space="preserve">Requires Docker; no public demo URL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retrieval gate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hybrid search (vector + Postgres full-text, reciprocal rank fusion) with a topic-keyword found rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plain similarity threshold (the original plan); reranker / LLM relevance grader</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured on real embeddings: the weakest correct answer scored 0.27 while the strongest wrong match for an out-of-scope question scored 0.42, so no threshold separates them. A topic keyword either occurs in the knowledge base or it doesn't. Hybrid+RRF is the industry-standard pattern; eval: 14/14 found, 5/5 gaps rejected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second index and ~ms per search; the found rule's frame-verb exclusion is a heuristic. Production upgrade: a reranker or LLM relevance grader (calibrated 'does this chunk answer the question?' scores) at ~200-400 ms per search</t>
   </si>
 </sst>
 </file>
@@ -4973,7 +4991,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -5294,6 +5312,29 @@
         <v>69</v>
       </c>
     </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>380</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>381</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>382</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>383</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>384</v>
+      </c>
+      <c r="F17" s="33" t="s">
+        <v>385</v>
+      </c>
+      <c r="G17" s="35" t="s">
+        <v>103</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Mark PR-05 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="387">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">Why hybrid instead of a similarity threshold (measured: 0.27 correct vs 0.42 wrong); RRF; what a 'topic keyword' is and why frame verbs are excluded; sources come from retrieval not the LLM; reranker as the production next step</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #6. Hybrid search (D-13) replaced the planned threshold after measurement. Eval 15/15 found, 6/6 gaps; pgTAP tests added.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-06</t>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t xml:space="preserve">Why these 3 tools; errors as tool results so the model can recover; validation at tool boundary; idempotency; prompt-injection limits via tool scope</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-07</t>
@@ -2327,7 +2330,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2363,7 +2366,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>4.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2372,7 +2375,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.166666666666667</v>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2390,7 +2393,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2580,7 +2583,7 @@
       </c>
       <c r="D28" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A28,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3074,13 +3077,15 @@
         <v>19</v>
       </c>
       <c r="M9" s="37" t="s">
-        <v>110</v>
+        <v>29</v>
       </c>
       <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
         <v>3</v>
       </c>
-      <c r="O9" s="38"/>
+      <c r="O9" s="38" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
@@ -3120,7 +3125,7 @@
         <v>19</v>
       </c>
       <c r="M10" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
@@ -3130,13 +3135,13 @@
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D11" s="40" t="s">
         <v>32</v>
@@ -3145,16 +3150,16 @@
         <v>72</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G11" s="33" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I11" s="33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J11" s="35" t="s">
         <v>111</v>
@@ -3166,7 +3171,7 @@
         <v>20</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
@@ -3176,13 +3181,13 @@
     </row>
     <row r="12" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>33</v>
@@ -3191,19 +3196,19 @@
         <v>72</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J12" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K12" s="36" t="n">
         <v>3</v>
@@ -3212,7 +3217,7 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
@@ -3222,13 +3227,13 @@
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>34</v>
@@ -3237,19 +3242,19 @@
         <v>72</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J13" s="35" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K13" s="36" t="n">
         <v>4</v>
@@ -3258,7 +3263,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3268,13 +3273,13 @@
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>35</v>
@@ -3283,16 +3288,16 @@
         <v>72</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J14" s="35" t="s">
         <v>95</v>
@@ -3304,7 +3309,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3314,13 +3319,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3329,16 +3334,16 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J15" s="35" t="s">
         <v>111</v>
@@ -3350,7 +3355,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3360,34 +3365,34 @@
     </row>
     <row r="16" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="J16" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K16" s="36" t="n">
         <v>2</v>
@@ -3396,7 +3401,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3406,13 +3411,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3421,19 +3426,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3442,7 +3447,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3452,13 +3457,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3467,19 +3472,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3488,7 +3493,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3498,7 +3503,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B19" s="47"/>
       <c r="C19" s="47"/>
@@ -3523,7 +3528,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K20" s="16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -3600,58 +3605,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F5" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E5,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3664,22 +3669,22 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E6,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3692,22 +3697,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F7" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E7,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3720,19 +3725,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
@@ -3746,19 +3751,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
@@ -3772,19 +3777,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
@@ -3798,19 +3803,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
@@ -3824,19 +3829,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
@@ -3850,19 +3855,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F13" s="35" t="s">
         <v>111</v>
@@ -3878,19 +3883,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
@@ -3904,19 +3909,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
@@ -3930,13 +3935,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -3949,7 +3954,7 @@
       </c>
       <c r="G16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E16,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E16,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3958,13 +3963,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -3973,11 +3978,11 @@
         <v>103</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3986,13 +3991,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4005,7 +4010,7 @@
       </c>
       <c r="G18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E18,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4014,13 +4019,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4040,13 +4045,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4055,7 +4060,7 @@
         <v>111</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4068,13 +4073,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4094,13 +4099,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4122,13 +4127,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4137,7 +4142,7 @@
         <v>111</v>
       </c>
       <c r="F23" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4150,13 +4155,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4176,13 +4181,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4204,19 +4209,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F26" s="35"/>
       <c r="G26" s="49" t="str">
@@ -4230,22 +4235,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E27" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F27" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4258,19 +4263,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E28" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F28" s="35" t="s">
         <v>111</v>
@@ -4286,22 +4291,22 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F29" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E29,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4314,19 +4319,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>95</v>
@@ -4342,13 +4347,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4357,7 +4362,7 @@
         <v>95</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4370,19 +4375,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
@@ -4396,19 +4401,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
@@ -4422,19 +4427,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F34" s="35" t="s">
         <v>103</v>
@@ -4450,19 +4455,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4476,19 +4481,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4502,19 +4507,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4528,19 +4533,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4554,19 +4559,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F39" s="35" t="s">
         <v>111</v>
@@ -4582,19 +4587,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4608,19 +4613,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F41" s="35"/>
       <c r="G41" s="49" t="str">
@@ -4634,13 +4639,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4649,7 +4654,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4662,13 +4667,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4688,22 +4693,22 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E44" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4716,19 +4721,19 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E45" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F45" s="35"/>
       <c r="G45" s="49" t="str">
@@ -4742,13 +4747,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4768,22 +4773,22 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4796,19 +4801,19 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E48" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F48" s="35" t="s">
         <v>69</v>
@@ -4824,13 +4829,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4850,19 +4855,19 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E50" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F50" s="35"/>
       <c r="G50" s="49" t="str">
@@ -4876,13 +4881,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -4891,7 +4896,7 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4904,16 +4909,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E52" s="35" t="s">
         <v>111</v>
@@ -4930,19 +4935,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5005,78 +5010,78 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G5" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5084,22 +5089,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5107,22 +5112,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5130,22 +5135,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5153,68 +5158,68 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G10" s="35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5222,22 +5227,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5245,22 +5250,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5268,22 +5273,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5291,22 +5296,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5314,22 +5319,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
Mark PR-06 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="388">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -445,7 +445,7 @@
     <t xml:space="preserve">Why these 3 tools; errors as tool results so the model can recover; validation at tool boundary; idempotency; prompt-injection limits via tool scope</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #7. Tools as atomic SQL functions; outcome_unknown for timed-out writes; prompt ordered for caching; R1 tested.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-07</t>
@@ -478,6 +478,9 @@
   </si>
   <si>
     <t xml:space="preserve">Hand-written loop vs AI SDK; server is source of truth for history; sliding window size &amp; cost; why tool traffic is not replayed; streaming protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-08</t>
@@ -2330,7 +2333,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2366,7 +2369,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$18,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2375,7 +2378,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.222222222222222</v>
+        <v>0.314814814814815</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2393,7 +2396,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2600,7 +2603,7 @@
       </c>
       <c r="D29" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$18,A29,'PR Plan'!$M$5:$M$18,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3125,13 +3128,15 @@
         <v>19</v>
       </c>
       <c r="M10" s="37" t="s">
-        <v>118</v>
+        <v>29</v>
       </c>
       <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
         <v>11</v>
       </c>
-      <c r="O10" s="38"/>
+      <c r="O10" s="38" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
@@ -3171,7 +3176,7 @@
         <v>20</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
@@ -3181,13 +3186,13 @@
     </row>
     <row r="12" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D12" s="41" t="s">
         <v>33</v>
@@ -3196,16 +3201,16 @@
         <v>72</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G12" s="33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H12" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J12" s="35" t="s">
         <v>119</v>
@@ -3217,7 +3222,7 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
@@ -3227,13 +3232,13 @@
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>34</v>
@@ -3242,19 +3247,19 @@
         <v>72</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G13" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J13" s="35" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K13" s="36" t="n">
         <v>4</v>
@@ -3263,7 +3268,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3273,13 +3278,13 @@
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>35</v>
@@ -3288,16 +3293,16 @@
         <v>72</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J14" s="35" t="s">
         <v>95</v>
@@ -3309,7 +3314,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3319,13 +3324,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3334,16 +3339,16 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J15" s="35" t="s">
         <v>111</v>
@@ -3355,7 +3360,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3365,31 +3370,31 @@
     </row>
     <row r="16" customFormat="false" ht="96.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>119</v>
@@ -3401,7 +3406,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3411,13 +3416,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3426,19 +3431,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3447,7 +3452,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3457,13 +3462,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3472,19 +3477,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3493,7 +3498,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3503,7 +3508,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B19" s="47"/>
       <c r="C19" s="47"/>
@@ -3528,7 +3533,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K20" s="16" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3605,55 +3610,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E5" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F5" s="35" t="s">
         <v>119</v>
@@ -3669,19 +3674,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F6" s="35" t="s">
         <v>119</v>
@@ -3697,19 +3702,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E7" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F7" s="35" t="s">
         <v>119</v>
@@ -3725,19 +3730,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
@@ -3751,19 +3756,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
@@ -3777,19 +3782,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
@@ -3803,19 +3808,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E11" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
@@ -3829,19 +3834,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
@@ -3855,19 +3860,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F13" s="35" t="s">
         <v>111</v>
@@ -3883,19 +3888,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
@@ -3909,19 +3914,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E15" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
@@ -3935,13 +3940,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -3963,13 +3968,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -3978,7 +3983,7 @@
         <v>103</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E17,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -3991,13 +3996,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4019,13 +4024,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4036,7 +4041,7 @@
       <c r="F19" s="35"/>
       <c r="G19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E19,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E19,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4045,13 +4050,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4060,11 +4065,11 @@
         <v>111</v>
       </c>
       <c r="F20" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E20,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4073,13 +4078,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4090,7 +4095,7 @@
       <c r="F21" s="35"/>
       <c r="G21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E21,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E21,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4099,13 +4104,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4118,7 +4123,7 @@
       </c>
       <c r="G22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E22,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E22,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4127,13 +4132,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4142,11 +4147,11 @@
         <v>111</v>
       </c>
       <c r="F23" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E23,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4155,13 +4160,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4172,7 +4177,7 @@
       <c r="F24" s="35"/>
       <c r="G24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E24,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E24,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4181,13 +4186,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4200,7 +4205,7 @@
       </c>
       <c r="G25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E25,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E25,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4209,13 +4214,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4235,13 +4240,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4250,7 +4255,7 @@
         <v>119</v>
       </c>
       <c r="F27" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E27,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4263,13 +4268,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4291,19 +4296,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E29" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F29" s="35" t="s">
         <v>119</v>
@@ -4319,19 +4324,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>95</v>
@@ -4347,13 +4352,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4362,7 +4367,7 @@
         <v>95</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E31,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4375,19 +4380,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
@@ -4401,19 +4406,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
@@ -4427,19 +4432,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F34" s="35" t="s">
         <v>103</v>
@@ -4455,19 +4460,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4481,19 +4486,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4507,19 +4512,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4533,19 +4538,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4559,19 +4564,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F39" s="35" t="s">
         <v>111</v>
@@ -4587,19 +4592,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4613,19 +4618,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F41" s="35"/>
       <c r="G41" s="49" t="str">
@@ -4639,13 +4644,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4654,11 +4659,11 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E42,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4667,13 +4672,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4684,7 +4689,7 @@
       <c r="F43" s="35"/>
       <c r="G43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E43,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E43,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4693,13 +4698,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4708,7 +4713,7 @@
         <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E44,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4721,13 +4726,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4747,13 +4752,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4773,22 +4778,22 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E47" s="35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E47,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4801,19 +4806,19 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E48" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F48" s="35" t="s">
         <v>69</v>
@@ -4829,13 +4834,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4855,13 +4860,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -4881,13 +4886,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -4896,11 +4901,11 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E51,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4909,16 +4914,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E52" s="35" t="s">
         <v>111</v>
@@ -4926,7 +4931,7 @@
       <c r="F52" s="35"/>
       <c r="G52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$18,MATCH(E52,'PR Plan'!$A$5:$A$18,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$18,MATCH(E52,'PR Plan'!$A$5:$A$18,0)),"-")</f>
@@ -4935,19 +4940,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5010,55 +5015,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5066,22 +5071,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5089,22 +5094,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5112,22 +5117,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5135,22 +5140,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5158,22 +5163,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5181,45 +5186,45 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G11" s="35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5227,22 +5232,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5250,22 +5255,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5273,22 +5278,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5296,22 +5301,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5319,22 +5324,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>

</xml_diff>

<commit_message>
Mark PR-07 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="406">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -480,10 +480,7 @@
     <t xml:space="preserve">Hand-written loop vs AI SDK; server is source of truth for history; sliding window size &amp; cost; why tool traffic is not replayed; streaming protocol</t>
   </si>
   <si>
-    <t xml:space="preserve">In review</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PR #8 open. Three review rounds; retry lease, one turn per conversation, integration tests.</t>
+    <t xml:space="preserve">Merged: PR #8. Three review rounds: retry lease, one turn per conversation, integration tests.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-08</t>
@@ -1625,24 +1622,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1674,7 +1675,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1686,11 +1687,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1698,51 +1699,51 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1835,7 +1836,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="26">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -1973,14 +1974,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFBBF7D0"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDDD6FE"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -2369,456 +2362,456 @@
   <dimension ref="A1:E43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <f aca="false">COUNTA('PR Plan'!$A$5:$A$19)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"In progress")+COUNTIF('PR Plan'!$M$5:$M$19,"In review")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"In progress")+COUNTIF('PR Plan'!$M$5:$M$19,"In review")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <f aca="false">SUM('PR Plan'!$K$5:$K$19)</f>
         <v>29.5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.288135593220339</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+        <v>0.372881355932203</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <f aca="false">COUNTA('Story Coverage'!$A$5:$A$1000)</f>
         <v>50</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="6" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$D:$D,"Must")</f>
         <v>39</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A18)</f>
         <v>8.5</v>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">B18-C18</f>
         <v>-0.5</v>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A18)</f>
         <v>6</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A19)</f>
         <v>11.5</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">B19-C19</f>
         <v>0.5</v>
       </c>
-      <c r="E19" s="11" t="n">
+      <c r="E19" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A19)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A20)</f>
         <v>8</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="11" t="n">
         <f aca="false">B20-C20</f>
         <v>-3</v>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A20)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A21)</f>
         <v>1.5</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">B21-C21</f>
         <v>-1.5</v>
       </c>
-      <c r="E21" s="11" t="n">
+      <c r="E21" s="12" t="n">
         <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A21)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="14" t="n">
         <f aca="false">SUM(B18:B21)</f>
         <v>25</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="C22" s="14" t="n">
         <f aca="false">SUM(C18:C21)</f>
         <v>29.5</v>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="14" t="n">
         <f aca="false">B22-C22</f>
         <v>-4.5</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="15" t="n">
         <f aca="false">SUM(E18:E21)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A27)</f>
         <v>2.5</v>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C27" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A27)</f>
         <v>3</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A27,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A28)</f>
         <v>3.5</v>
       </c>
-      <c r="C28" s="17" t="n">
+      <c r="C28" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A28)</f>
         <v>2</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A28,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A29)</f>
         <v>5</v>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C29" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A29)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A29,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A30)</f>
         <v>3</v>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C30" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A30)</f>
         <v>1</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A30,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A31)</f>
         <v>4</v>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C31" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A31)</f>
         <v>1</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A31,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A32)</f>
         <v>8</v>
       </c>
-      <c r="C32" s="17" t="n">
+      <c r="C32" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A32)</f>
         <v>4</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A33)</f>
         <v>1.5</v>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C33" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A33)</f>
         <v>1</v>
       </c>
-      <c r="D33" s="17" t="n">
+      <c r="D33" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A33,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="24" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="10" t="n">
+      <c r="B34" s="11" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A34)</f>
         <v>2</v>
       </c>
-      <c r="C34" s="17" t="n">
+      <c r="C34" s="18" t="n">
         <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A34)</f>
         <v>1</v>
       </c>
-      <c r="D34" s="17" t="n">
+      <c r="D34" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A34,'PR Plan'!$M$5:$M$19,"Done")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B37" s="27" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="27" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="B38" s="27" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="27" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="29" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="27" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="29" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="B41" s="27" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="29" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" s="27" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="29" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="B43" s="27" t="s">
         <v>52</v>
       </c>
     </row>
@@ -2847,841 +2840,841 @@
   <dimension ref="A1:O21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="31" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="G4" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="H4" s="30" t="s">
+      <c r="H4" s="31" t="s">
         <v>61</v>
       </c>
-      <c r="I4" s="30" t="s">
+      <c r="I4" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="J4" s="30" t="s">
+      <c r="J4" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="K4" s="30" t="s">
+      <c r="K4" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="L4" s="30" t="s">
+      <c r="L4" s="31" t="s">
         <v>65</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="M4" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="N4" s="30" t="s">
+      <c r="N4" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="O4" s="30" t="s">
+      <c r="O4" s="31" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="33" t="s">
+      <c r="D5" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="33" t="s">
         <v>73</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="I5" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="J5" s="34" t="s">
+      <c r="J5" s="35" t="s">
         <v>77</v>
       </c>
-      <c r="K5" s="35" t="n">
+      <c r="K5" s="36" t="n">
         <v>0.5</v>
       </c>
-      <c r="L5" s="34" t="s">
+      <c r="L5" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="36" t="s">
+      <c r="M5" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N5" s="34" t="n">
+      <c r="N5" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A5)</f>
         <v>0</v>
       </c>
-      <c r="O5" s="37" t="s">
+      <c r="O5" s="38" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="33" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="J6" s="34" t="s">
+      <c r="J6" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="K6" s="35" t="n">
+      <c r="K6" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L6" s="34" t="s">
+      <c r="L6" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M6" s="36" t="s">
+      <c r="M6" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N6" s="34" t="n">
+      <c r="N6" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A6)</f>
         <v>1</v>
       </c>
-      <c r="O6" s="37" t="s">
+      <c r="O6" s="38" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="34" t="s">
+      <c r="E7" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="F7" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="H7" s="32" t="s">
+      <c r="H7" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="I7" s="32" t="s">
+      <c r="I7" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="J7" s="34" t="s">
+      <c r="J7" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="K7" s="35" t="n">
+      <c r="K7" s="36" t="n">
         <v>0.5</v>
       </c>
-      <c r="L7" s="34" t="s">
+      <c r="L7" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M7" s="36" t="s">
+      <c r="M7" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N7" s="34" t="n">
+      <c r="N7" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A7)</f>
         <v>0</v>
       </c>
-      <c r="O7" s="37" t="s">
+      <c r="O7" s="38" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="33" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="I8" s="33" t="s">
         <v>101</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="J8" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="K8" s="35" t="n">
+      <c r="K8" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="L8" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="36" t="s">
+      <c r="M8" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N8" s="34" t="n">
+      <c r="N8" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A8)</f>
         <v>2</v>
       </c>
-      <c r="O8" s="37" t="s">
+      <c r="O8" s="38" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="34" t="s">
+      <c r="E9" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="F9" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="H9" s="32" t="s">
+      <c r="H9" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="I9" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="J9" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="K9" s="35" t="n">
+      <c r="K9" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L9" s="34" t="s">
+      <c r="L9" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M9" s="36" t="s">
+      <c r="M9" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N9" s="34" t="n">
+      <c r="N9" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A9)</f>
         <v>3</v>
       </c>
-      <c r="O9" s="37" t="s">
+      <c r="O9" s="38" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="34" t="s">
+      <c r="E10" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="H10" s="32" t="s">
+      <c r="H10" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="I10" s="32" t="s">
+      <c r="I10" s="33" t="s">
         <v>117</v>
       </c>
-      <c r="J10" s="34" t="s">
+      <c r="J10" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="K10" s="35" t="n">
+      <c r="K10" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="L10" s="34" t="s">
+      <c r="L10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="M10" s="36" t="s">
+      <c r="M10" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="N10" s="34" t="n">
+      <c r="N10" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A10)</f>
         <v>11</v>
       </c>
-      <c r="O10" s="37" t="s">
+      <c r="O10" s="38" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="187.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="C11" s="32" t="s">
+      <c r="C11" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="D11" s="39" t="s">
+      <c r="D11" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="34" t="s">
+      <c r="E11" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="G11" s="32" t="s">
+      <c r="G11" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="H11" s="32" t="s">
+      <c r="H11" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="I11" s="32" t="s">
+      <c r="I11" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="J11" s="34" t="s">
+      <c r="J11" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="K11" s="35" t="n">
+      <c r="K11" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="L11" s="34" t="s">
+      <c r="L11" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M11" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="N11" s="34" t="n">
+      <c r="M11" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A11)</f>
         <v>6</v>
       </c>
-      <c r="O11" s="37" t="s">
+      <c r="O11" s="38" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="279" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
+      <c r="B12" s="33" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="C12" s="33" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="D12" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="D12" s="40" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F12" s="32" t="s">
+      <c r="G12" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="H12" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="I12" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="I12" s="32" t="s">
+      <c r="J12" s="35" t="s">
+        <v>119</v>
+      </c>
+      <c r="K12" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="M12" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="K12" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="M12" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N12" s="34" t="n">
+      <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
         <v>6</v>
       </c>
-      <c r="O12" s="37"/>
+      <c r="O12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="C13" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="D13" s="42" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="D13" s="41" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="32" t="s">
+      <c r="G13" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="H13" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="I13" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="J13" s="35" t="s">
         <v>142</v>
       </c>
-      <c r="J13" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="K13" s="35" t="n">
+      <c r="K13" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="L13" s="34" t="s">
+      <c r="L13" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N13" s="34" t="n">
+      <c r="M13" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
         <v>8</v>
       </c>
-      <c r="O13" s="37"/>
+      <c r="O13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
+      <c r="A14" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="C14" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="D14" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="D14" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F14" s="32" t="s">
+      <c r="G14" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="H14" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="H14" s="32" t="s">
+      <c r="I14" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="I14" s="32" t="s">
-        <v>150</v>
-      </c>
-      <c r="J14" s="34" t="s">
+      <c r="J14" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="K14" s="35" t="n">
+      <c r="K14" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L14" s="34" t="s">
+      <c r="L14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="M14" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N14" s="34" t="n">
+      <c r="M14" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
         <v>4</v>
       </c>
-      <c r="O14" s="37"/>
+      <c r="O14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="C15" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="D15" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="33" t="s">
         <v>153</v>
       </c>
-      <c r="D15" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F15" s="32" t="s">
+      <c r="G15" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="G15" s="32" t="s">
+      <c r="H15" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="H15" s="32" t="s">
+      <c r="I15" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="I15" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="J15" s="34" t="s">
+      <c r="J15" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="K15" s="35" t="n">
+      <c r="K15" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L15" s="34" t="s">
+      <c r="L15" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M15" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N15" s="34" t="n">
+      <c r="M15" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
         <v>3</v>
       </c>
-      <c r="O15" s="37"/>
+      <c r="O15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="C16" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="D16" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="35" t="s">
         <v>160</v>
       </c>
-      <c r="D16" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="34" t="s">
+      <c r="F16" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="G16" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="G16" s="32" t="s">
+      <c r="H16" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="H16" s="32" t="s">
+      <c r="I16" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="I16" s="32" t="s">
-        <v>165</v>
-      </c>
-      <c r="J16" s="34" t="s">
+      <c r="J16" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="K16" s="35" t="n">
+      <c r="K16" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L16" s="34" t="s">
+      <c r="L16" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="M16" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N16" s="34" t="n">
+      <c r="M16" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
         <v>3</v>
       </c>
-      <c r="O16" s="37"/>
+      <c r="O16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="B17" s="32" t="s">
+      <c r="C17" s="33" t="s">
         <v>167</v>
       </c>
-      <c r="C17" s="32" t="s">
+      <c r="D17" s="44" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="33" t="s">
         <v>168</v>
       </c>
-      <c r="D17" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F17" s="32" t="s">
+      <c r="G17" s="33" t="s">
         <v>169</v>
       </c>
-      <c r="G17" s="32" t="s">
+      <c r="H17" s="33" t="s">
         <v>170</v>
       </c>
-      <c r="H17" s="32" t="s">
+      <c r="I17" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="J17" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="J17" s="34" t="s">
-        <v>173</v>
-      </c>
-      <c r="K17" s="35" t="n">
+      <c r="K17" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="L17" s="34" t="s">
+      <c r="L17" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M17" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N17" s="34" t="n">
+      <c r="M17" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
         <v>1</v>
       </c>
-      <c r="O17" s="37"/>
+      <c r="O17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
+      <c r="A18" s="32" t="s">
+        <v>173</v>
+      </c>
+      <c r="B18" s="33" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="32" t="s">
+      <c r="C18" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="D18" s="45" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="33" t="s">
         <v>176</v>
       </c>
-      <c r="D18" s="44" t="s">
-        <v>37</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>72</v>
-      </c>
-      <c r="F18" s="32" t="s">
+      <c r="G18" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="G18" s="32" t="s">
+      <c r="H18" s="33" t="s">
         <v>178</v>
       </c>
-      <c r="H18" s="32" t="s">
+      <c r="I18" s="33" t="s">
         <v>179</v>
       </c>
-      <c r="I18" s="32" t="s">
+      <c r="J18" s="35" t="s">
         <v>180</v>
       </c>
-      <c r="J18" s="34" t="s">
-        <v>181</v>
-      </c>
-      <c r="K18" s="35" t="n">
+      <c r="K18" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="L18" s="34" t="s">
+      <c r="L18" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M18" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N18" s="34" t="n">
+      <c r="M18" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
         <v>0</v>
       </c>
-      <c r="O18" s="37"/>
+      <c r="O18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="32" t="s">
+        <v>181</v>
+      </c>
+      <c r="B19" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B19" s="32" t="s">
+      <c r="C19" s="33" t="s">
         <v>183</v>
       </c>
-      <c r="C19" s="32" t="s">
+      <c r="D19" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="F19" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="D19" s="42" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="F19" s="32" t="s">
+      <c r="G19" s="33" t="s">
         <v>185</v>
       </c>
-      <c r="G19" s="32" t="s">
+      <c r="H19" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="H19" s="32" t="s">
+      <c r="I19" s="33" t="s">
         <v>187</v>
       </c>
-      <c r="I19" s="32" t="s">
+      <c r="J19" s="35" t="s">
         <v>188</v>
       </c>
-      <c r="J19" s="34" t="s">
-        <v>189</v>
-      </c>
-      <c r="K19" s="35" t="n">
+      <c r="K19" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="L19" s="34" t="s">
+      <c r="L19" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="M19" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="N19" s="34" t="n">
+      <c r="M19" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
-      <c r="O19" s="37" t="s">
+      <c r="O19" s="38" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="46" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="45" t="s">
-        <v>191</v>
-      </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="47" t="n">
+      <c r="B20" s="47"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="47"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="47"/>
+      <c r="J20" s="47"/>
+      <c r="K20" s="48" t="n">
         <f aca="false">SUM(K5:K19)</f>
         <v>29.5</v>
       </c>
-      <c r="L20" s="46"/>
-      <c r="M20" s="46"/>
-      <c r="N20" s="45" t="n">
+      <c r="L20" s="47"/>
+      <c r="M20" s="47"/>
+      <c r="N20" s="46" t="n">
         <f aca="false">SUM(N5:N19)</f>
         <v>50</v>
       </c>
-      <c r="O20" s="46"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K21" s="15" t="s">
-        <v>192</v>
+      <c r="O20" s="47"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K21" s="16" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:O19"/>
   <conditionalFormatting sqref="M5:M19">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:E19">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
       <formula>"Should"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L19">
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="25">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M5="Done"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3718,1398 +3711,1398 @@
   <dimension ref="A1:H54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="31" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>196</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="D4" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="31" t="s">
         <v>197</v>
       </c>
-      <c r="D4" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>198</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="G4" s="31" t="s">
         <v>199</v>
       </c>
-      <c r="G4" s="30" t="s">
+      <c r="H4" s="31" t="s">
         <v>200</v>
       </c>
-      <c r="H4" s="30" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="B5" s="33" t="s">
         <v>202</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="C5" s="33" t="s">
         <v>203</v>
       </c>
-      <c r="C5" s="32" t="s">
-        <v>204</v>
-      </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F5" s="34" t="s">
+      <c r="E5" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="G5" s="48" t="str">
+      <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H5" s="48" t="str">
+      <c r="H5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" s="33" t="s">
         <v>205</v>
       </c>
-      <c r="B6" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C6" s="32" t="s">
-        <v>206</v>
-      </c>
-      <c r="D6" s="34" t="s">
+      <c r="D6" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F6" s="34" t="s">
+      <c r="E6" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="G6" s="48" t="str">
+      <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H6" s="48" t="str">
+      <c r="H6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C7" s="33" t="s">
         <v>207</v>
       </c>
-      <c r="B7" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C7" s="32" t="s">
-        <v>208</v>
-      </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E7" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F7" s="34" t="s">
+      <c r="E7" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="G7" s="48" t="str">
+      <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H7" s="48" t="str">
+      <c r="H7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="B8" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="33" t="s">
         <v>209</v>
       </c>
-      <c r="B8" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C8" s="32" t="s">
-        <v>210</v>
-      </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E8" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" s="34"/>
-      <c r="G8" s="48" t="str">
+      <c r="E8" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="35"/>
+      <c r="G8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H8" s="48" t="str">
+      <c r="H8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>210</v>
+      </c>
+      <c r="B9" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="33" t="s">
         <v>211</v>
       </c>
-      <c r="B9" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C9" s="32" t="s">
+      <c r="D9" s="35" t="s">
         <v>212</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="48" t="str">
+      <c r="E9" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F9" s="35"/>
+      <c r="G9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H9" s="48" t="str">
+      <c r="H9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="B10" s="33" t="s">
         <v>214</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="C10" s="33" t="s">
         <v>215</v>
       </c>
-      <c r="C10" s="32" t="s">
-        <v>216</v>
-      </c>
-      <c r="D10" s="34" t="s">
+      <c r="D10" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F10" s="34"/>
-      <c r="G10" s="48" t="str">
+      <c r="E10" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="35"/>
+      <c r="G10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H10" s="48" t="str">
+      <c r="H10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="C11" s="33" t="s">
         <v>217</v>
       </c>
-      <c r="B11" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>218</v>
-      </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E11" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="48" t="str">
+      <c r="E11" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F11" s="35"/>
+      <c r="G11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H11" s="48" t="str">
+      <c r="H11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" s="33" t="s">
         <v>219</v>
       </c>
-      <c r="B12" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C12" s="32" t="s">
-        <v>220</v>
-      </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E12" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F12" s="34"/>
-      <c r="G12" s="48" t="str">
+      <c r="E12" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F12" s="35"/>
+      <c r="G12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H12" s="48" t="str">
+      <c r="H12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="32" t="s">
+        <v>220</v>
+      </c>
+      <c r="B13" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="C13" s="33" t="s">
         <v>221</v>
       </c>
-      <c r="B13" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C13" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="D13" s="34" t="s">
+      <c r="D13" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F13" s="34" t="s">
+      <c r="E13" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F13" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="48" t="str">
+      <c r="G13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H13" s="48" t="str">
+      <c r="H13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="C14" s="33" t="s">
         <v>223</v>
       </c>
-      <c r="B14" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C14" s="32" t="s">
-        <v>224</v>
-      </c>
-      <c r="D14" s="34" t="s">
+      <c r="D14" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E14" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F14" s="34"/>
-      <c r="G14" s="48" t="str">
+      <c r="E14" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F14" s="35"/>
+      <c r="G14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H14" s="48" t="str">
+      <c r="H14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="C15" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="B15" s="32" t="s">
-        <v>215</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>226</v>
-      </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F15" s="34"/>
-      <c r="G15" s="48" t="str">
+      <c r="E15" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F15" s="35"/>
+      <c r="G15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H15" s="48" t="str">
+      <c r="H15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" s="33" t="s">
         <v>227</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="C16" s="33" t="s">
         <v>228</v>
       </c>
-      <c r="C16" s="32" t="s">
-        <v>229</v>
-      </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="34" t="s">
+      <c r="F16" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="G16" s="48" t="str">
+      <c r="G16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E16,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H16" s="48" t="str">
+      <c r="H16" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E16,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>229</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="C17" s="33" t="s">
         <v>230</v>
       </c>
-      <c r="B17" s="32" t="s">
-        <v>228</v>
-      </c>
-      <c r="C17" s="32" t="s">
-        <v>231</v>
-      </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="F17" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="G17" s="48" t="str">
+      <c r="F17" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="G17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E17,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H17" s="48" t="str">
+      <c r="H17" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E17,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="32" t="s">
+        <v>231</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="C18" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>228</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>233</v>
-      </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="F18" s="34" t="s">
+      <c r="F18" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G18" s="48" t="str">
+      <c r="G18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E18,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H18" s="48" t="str">
+      <c r="H18" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E18,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="32" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>227</v>
+      </c>
+      <c r="C19" s="33" t="s">
         <v>234</v>
       </c>
-      <c r="B19" s="32" t="s">
-        <v>228</v>
-      </c>
-      <c r="C19" s="32" t="s">
-        <v>235</v>
-      </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E19" s="34" t="s">
+      <c r="E19" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="34"/>
-      <c r="G19" s="48" t="str">
+      <c r="F19" s="35"/>
+      <c r="G19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E19,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H19" s="48" t="str">
+      <c r="H19" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E19,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="32" t="s">
+        <v>235</v>
+      </c>
+      <c r="B20" s="33" t="s">
         <v>236</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="C20" s="33" t="s">
         <v>237</v>
       </c>
-      <c r="C20" s="32" t="s">
-        <v>238</v>
-      </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="34" t="s">
+      <c r="E20" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F20" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="G20" s="48" t="str">
+      <c r="F20" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="G20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E20,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H20" s="48" t="str">
+      <c r="H20" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E20,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="31" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="32" t="s">
+        <v>238</v>
+      </c>
+      <c r="B21" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C21" s="33" t="s">
         <v>239</v>
       </c>
-      <c r="B21" s="32" t="s">
-        <v>237</v>
-      </c>
-      <c r="C21" s="32" t="s">
-        <v>240</v>
-      </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E21" s="34" t="s">
+      <c r="E21" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F21" s="34"/>
-      <c r="G21" s="48" t="str">
+      <c r="F21" s="35"/>
+      <c r="G21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E21,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H21" s="48" t="str">
+      <c r="H21" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E21,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="B22" s="33" t="s">
+        <v>236</v>
+      </c>
+      <c r="C22" s="33" t="s">
         <v>241</v>
       </c>
-      <c r="B22" s="32" t="s">
-        <v>237</v>
-      </c>
-      <c r="C22" s="32" t="s">
-        <v>242</v>
-      </c>
-      <c r="D22" s="34" t="s">
+      <c r="D22" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E22" s="34" t="s">
+      <c r="E22" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F22" s="34" t="s">
+      <c r="F22" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="G22" s="48" t="str">
+      <c r="G22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E22,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H22" s="48" t="str">
+      <c r="H22" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E22,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="31" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="B23" s="33" t="s">
         <v>243</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="C23" s="33" t="s">
         <v>244</v>
       </c>
-      <c r="C23" s="32" t="s">
-        <v>245</v>
-      </c>
-      <c r="D23" s="34" t="s">
+      <c r="D23" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="34" t="s">
+      <c r="E23" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F23" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="G23" s="48" t="str">
+      <c r="F23" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="G23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E23,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H23" s="48" t="str">
+      <c r="H23" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E23,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="31" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="32" t="s">
+        <v>245</v>
+      </c>
+      <c r="B24" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="C24" s="33" t="s">
         <v>246</v>
       </c>
-      <c r="B24" s="32" t="s">
-        <v>244</v>
-      </c>
-      <c r="C24" s="32" t="s">
-        <v>247</v>
-      </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E24" s="34" t="s">
+      <c r="E24" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F24" s="34"/>
-      <c r="G24" s="48" t="str">
+      <c r="F24" s="35"/>
+      <c r="G24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E24,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H24" s="48" t="str">
+      <c r="H24" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E24,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="B25" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="C25" s="33" t="s">
         <v>248</v>
       </c>
-      <c r="B25" s="32" t="s">
-        <v>244</v>
-      </c>
-      <c r="C25" s="32" t="s">
-        <v>249</v>
-      </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="34" t="s">
+      <c r="E25" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="G25" s="48" t="str">
+      <c r="G25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E25,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H25" s="48" t="str">
+      <c r="H25" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E25,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="31" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="B26" s="33" t="s">
         <v>250</v>
       </c>
-      <c r="B26" s="32" t="s">
+      <c r="C26" s="33" t="s">
         <v>251</v>
       </c>
-      <c r="C26" s="32" t="s">
-        <v>252</v>
-      </c>
-      <c r="D26" s="34" t="s">
+      <c r="D26" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E26" s="34" t="s">
+      <c r="E26" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F26" s="34"/>
-      <c r="G26" s="48" t="str">
+      <c r="F26" s="35"/>
+      <c r="G26" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E26,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H26" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H26" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E26,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="31" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="32" t="s">
+        <v>252</v>
+      </c>
+      <c r="B27" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="C27" s="33" t="s">
         <v>253</v>
       </c>
-      <c r="B27" s="32" t="s">
-        <v>251</v>
-      </c>
-      <c r="C27" s="32" t="s">
-        <v>254</v>
-      </c>
-      <c r="D27" s="34" t="s">
+      <c r="D27" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E27" s="34" t="s">
+      <c r="E27" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F27" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="G27" s="48" t="str">
+      <c r="F27" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="G27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E27,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H27" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H27" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E27,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="31" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="32" t="s">
+        <v>254</v>
+      </c>
+      <c r="B28" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="C28" s="33" t="s">
         <v>255</v>
       </c>
-      <c r="B28" s="32" t="s">
-        <v>251</v>
-      </c>
-      <c r="C28" s="32" t="s">
-        <v>256</v>
-      </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F28" s="34" t="s">
+      <c r="F28" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G28" s="48" t="str">
+      <c r="G28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E28,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H28" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H28" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E28,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="32" t="s">
+        <v>256</v>
+      </c>
+      <c r="B29" s="33" t="s">
+        <v>250</v>
+      </c>
+      <c r="C29" s="33" t="s">
         <v>257</v>
       </c>
-      <c r="B29" s="32" t="s">
-        <v>251</v>
-      </c>
-      <c r="C29" s="32" t="s">
-        <v>258</v>
-      </c>
-      <c r="D29" s="34" t="s">
+      <c r="D29" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E29" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F29" s="34" t="s">
+      <c r="E29" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="G29" s="48" t="str">
+      <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H29" s="48" t="str">
+      <c r="H29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="31" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="B30" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="C30" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="C30" s="32" t="s">
-        <v>261</v>
-      </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E30" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F30" s="34" t="s">
+      <c r="E30" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="F30" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="G30" s="48" t="str">
+      <c r="G30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H30" s="48" t="str">
+      <c r="H30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="32" t="s">
+        <v>261</v>
+      </c>
+      <c r="B31" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="33" t="s">
         <v>262</v>
       </c>
-      <c r="B31" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="C31" s="32" t="s">
-        <v>263</v>
-      </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="F31" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="G31" s="48" t="str">
+      <c r="F31" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E31,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H31" s="48" t="str">
+      <c r="H31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E31,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="31" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="32" t="s">
+        <v>263</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="C32" s="33" t="s">
         <v>264</v>
       </c>
-      <c r="B32" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="C32" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="D32" s="34" t="s">
+      <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E32" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F32" s="34"/>
-      <c r="G32" s="48" t="str">
+      <c r="E32" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="F32" s="35"/>
+      <c r="G32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H32" s="48" t="str">
+      <c r="H32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="31" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="B33" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="C33" s="33" t="s">
         <v>266</v>
       </c>
-      <c r="B33" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="C33" s="32" t="s">
-        <v>267</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E33" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F33" s="34"/>
-      <c r="G33" s="48" t="str">
+      <c r="D33" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="E33" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="F33" s="35"/>
+      <c r="G33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H33" s="48" t="str">
+      <c r="H33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="31" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>259</v>
+      </c>
+      <c r="C34" s="33" t="s">
         <v>268</v>
       </c>
-      <c r="B34" s="32" t="s">
-        <v>260</v>
-      </c>
-      <c r="C34" s="32" t="s">
-        <v>269</v>
-      </c>
-      <c r="D34" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E34" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="F34" s="34" t="s">
+      <c r="D34" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="E34" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="F34" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="G34" s="48" t="str">
+      <c r="G34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H34" s="48" t="str">
+      <c r="H34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="31" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="32" t="s">
+        <v>269</v>
+      </c>
+      <c r="B35" s="33" t="s">
         <v>270</v>
       </c>
-      <c r="B35" s="32" t="s">
+      <c r="C35" s="33" t="s">
         <v>271</v>
       </c>
-      <c r="C35" s="32" t="s">
-        <v>272</v>
-      </c>
-      <c r="D35" s="34" t="s">
+      <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E35" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="F35" s="34"/>
-      <c r="G35" s="48" t="str">
+      <c r="E35" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="F35" s="35"/>
+      <c r="G35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H35" s="48" t="str">
+      <c r="H35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="31" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32" t="s">
+        <v>272</v>
+      </c>
+      <c r="B36" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C36" s="33" t="s">
         <v>273</v>
       </c>
-      <c r="B36" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C36" s="32" t="s">
-        <v>274</v>
-      </c>
-      <c r="D36" s="34" t="s">
+      <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E36" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="F36" s="34"/>
-      <c r="G36" s="48" t="str">
+      <c r="E36" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="F36" s="35"/>
+      <c r="G36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H36" s="48" t="str">
+      <c r="H36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="31" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="32" t="s">
+        <v>274</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C37" s="33" t="s">
         <v>275</v>
       </c>
-      <c r="B37" s="32" t="s">
-        <v>271</v>
-      </c>
-      <c r="C37" s="32" t="s">
-        <v>276</v>
-      </c>
-      <c r="D37" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E37" s="34" t="s">
-        <v>151</v>
-      </c>
-      <c r="F37" s="34"/>
-      <c r="G37" s="48" t="str">
+      <c r="D37" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E37" s="35" t="s">
+        <v>150</v>
+      </c>
+      <c r="F37" s="35"/>
+      <c r="G37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H37" s="48" t="str">
+      <c r="H37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="31" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="32" t="s">
+        <v>276</v>
+      </c>
+      <c r="B38" s="33" t="s">
         <v>277</v>
       </c>
-      <c r="B38" s="32" t="s">
+      <c r="C38" s="33" t="s">
         <v>278</v>
       </c>
-      <c r="C38" s="32" t="s">
-        <v>279</v>
-      </c>
-      <c r="D38" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E38" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="F38" s="34"/>
-      <c r="G38" s="48" t="str">
+      <c r="D38" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E38" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="F38" s="35"/>
+      <c r="G38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H38" s="48" t="str">
+      <c r="H38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="31" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="32" t="s">
+        <v>279</v>
+      </c>
+      <c r="B39" s="33" t="s">
+        <v>277</v>
+      </c>
+      <c r="C39" s="33" t="s">
         <v>280</v>
       </c>
-      <c r="B39" s="32" t="s">
-        <v>278</v>
-      </c>
-      <c r="C39" s="32" t="s">
-        <v>281</v>
-      </c>
-      <c r="D39" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E39" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="F39" s="34" t="s">
+      <c r="D39" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E39" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="F39" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="48" t="str">
+      <c r="G39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H39" s="48" t="str">
+      <c r="H39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="31" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="32" t="s">
+        <v>281</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>277</v>
+      </c>
+      <c r="C40" s="33" t="s">
         <v>282</v>
       </c>
-      <c r="B40" s="32" t="s">
-        <v>278</v>
-      </c>
-      <c r="C40" s="32" t="s">
-        <v>283</v>
-      </c>
-      <c r="D40" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E40" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="F40" s="34"/>
-      <c r="G40" s="48" t="str">
+      <c r="D40" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="E40" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="F40" s="35"/>
+      <c r="G40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H40" s="48" t="str">
+      <c r="H40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="31" t="s">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="32" t="s">
+        <v>283</v>
+      </c>
+      <c r="B41" s="33" t="s">
         <v>284</v>
       </c>
-      <c r="B41" s="32" t="s">
+      <c r="C41" s="33" t="s">
         <v>285</v>
       </c>
-      <c r="C41" s="32" t="s">
-        <v>286</v>
-      </c>
-      <c r="D41" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E41" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="F41" s="34" t="s">
-        <v>158</v>
-      </c>
-      <c r="G41" s="48" t="str">
+      <c r="D41" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E41" s="35" t="s">
+        <v>181</v>
+      </c>
+      <c r="F41" s="35" t="s">
+        <v>157</v>
+      </c>
+      <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H41" s="48" t="str">
+      <c r="H41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="31" t="s">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="B42" s="33" t="s">
         <v>287</v>
       </c>
-      <c r="B42" s="32" t="s">
+      <c r="C42" s="33" t="s">
         <v>288</v>
       </c>
-      <c r="C42" s="32" t="s">
-        <v>289</v>
-      </c>
-      <c r="D42" s="34" t="s">
+      <c r="D42" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="34" t="s">
+      <c r="E42" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F42" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="G42" s="48" t="str">
+      <c r="F42" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H42" s="48" t="str">
+      <c r="H42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="31" t="s">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="32" t="s">
+        <v>289</v>
+      </c>
+      <c r="B43" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C43" s="33" t="s">
         <v>290</v>
       </c>
-      <c r="B43" s="32" t="s">
-        <v>288</v>
-      </c>
-      <c r="C43" s="32" t="s">
-        <v>291</v>
-      </c>
-      <c r="D43" s="34" t="s">
+      <c r="D43" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E43" s="34" t="s">
+      <c r="E43" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F43" s="34"/>
-      <c r="G43" s="48" t="str">
+      <c r="F43" s="35"/>
+      <c r="G43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E43,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H43" s="48" t="str">
+      <c r="H43" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E43,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="31" t="s">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="32" t="s">
+        <v>291</v>
+      </c>
+      <c r="B44" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C44" s="33" t="s">
         <v>292</v>
       </c>
-      <c r="B44" s="32" t="s">
-        <v>288</v>
-      </c>
-      <c r="C44" s="32" t="s">
-        <v>293</v>
-      </c>
-      <c r="D44" s="34" t="s">
+      <c r="D44" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E44" s="34" t="s">
+      <c r="E44" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F44" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="G44" s="48" t="str">
+      <c r="F44" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H44" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="31" t="s">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="32" t="s">
+        <v>293</v>
+      </c>
+      <c r="B45" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C45" s="33" t="s">
         <v>294</v>
       </c>
-      <c r="B45" s="32" t="s">
-        <v>288</v>
-      </c>
-      <c r="C45" s="32" t="s">
-        <v>295</v>
-      </c>
-      <c r="D45" s="34" t="s">
+      <c r="D45" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E45" s="34" t="s">
+      <c r="E45" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F45" s="34"/>
-      <c r="G45" s="48" t="str">
+      <c r="F45" s="35"/>
+      <c r="G45" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E45,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H45" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H45" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E45,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="31" t="s">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="32" t="s">
+        <v>295</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C46" s="33" t="s">
         <v>296</v>
       </c>
-      <c r="B46" s="32" t="s">
-        <v>288</v>
-      </c>
-      <c r="C46" s="32" t="s">
-        <v>297</v>
-      </c>
-      <c r="D46" s="34" t="s">
+      <c r="D46" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E46" s="34" t="s">
+      <c r="E46" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="F46" s="34"/>
-      <c r="G46" s="48" t="str">
+      <c r="F46" s="35"/>
+      <c r="G46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E46,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H46" s="48" t="str">
+      <c r="H46" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E46,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="31" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="B47" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="C47" s="33" t="s">
         <v>298</v>
       </c>
-      <c r="B47" s="32" t="s">
-        <v>288</v>
-      </c>
-      <c r="C47" s="32" t="s">
-        <v>299</v>
-      </c>
-      <c r="D47" s="34" t="s">
+      <c r="D47" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E47" s="34" t="s">
-        <v>128</v>
-      </c>
-      <c r="F47" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="G47" s="48" t="str">
+      <c r="E47" s="35" t="s">
+        <v>127</v>
+      </c>
+      <c r="F47" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H47" s="48" t="str">
+      <c r="H47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="31" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="32" t="s">
+        <v>299</v>
+      </c>
+      <c r="B48" s="33" t="s">
         <v>300</v>
       </c>
-      <c r="B48" s="32" t="s">
+      <c r="C48" s="33" t="s">
         <v>301</v>
       </c>
-      <c r="C48" s="32" t="s">
-        <v>302</v>
-      </c>
-      <c r="D48" s="34" t="s">
+      <c r="D48" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E48" s="34" t="s">
-        <v>136</v>
-      </c>
-      <c r="F48" s="34" t="s">
+      <c r="E48" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="F48" s="35" t="s">
         <v>69</v>
       </c>
-      <c r="G48" s="48" t="str">
+      <c r="G48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H48" s="48" t="str">
+      <c r="H48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="31" t="s">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="32" t="s">
+        <v>302</v>
+      </c>
+      <c r="B49" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="C49" s="33" t="s">
         <v>303</v>
       </c>
-      <c r="B49" s="32" t="s">
-        <v>301</v>
-      </c>
-      <c r="C49" s="32" t="s">
-        <v>304</v>
-      </c>
-      <c r="D49" s="34" t="s">
+      <c r="D49" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E49" s="34" t="s">
+      <c r="E49" s="35" t="s">
         <v>79</v>
       </c>
-      <c r="F49" s="34"/>
-      <c r="G49" s="48" t="str">
+      <c r="F49" s="35"/>
+      <c r="G49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E49,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H49" s="48" t="str">
+      <c r="H49" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E49,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="31" t="s">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="32" t="s">
+        <v>304</v>
+      </c>
+      <c r="B50" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="C50" s="33" t="s">
         <v>305</v>
       </c>
-      <c r="B50" s="32" t="s">
-        <v>301</v>
-      </c>
-      <c r="C50" s="32" t="s">
-        <v>306</v>
-      </c>
-      <c r="D50" s="34" t="s">
+      <c r="D50" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E50" s="34" t="s">
+      <c r="E50" s="35" t="s">
         <v>119</v>
       </c>
-      <c r="F50" s="34"/>
-      <c r="G50" s="48" t="str">
+      <c r="F50" s="35"/>
+      <c r="G50" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E50,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>In review</v>
-      </c>
-      <c r="H50" s="48" t="str">
+        <v>Done</v>
+      </c>
+      <c r="H50" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E50,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="31" t="s">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="32" t="s">
+        <v>306</v>
+      </c>
+      <c r="B51" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="C51" s="33" t="s">
         <v>307</v>
       </c>
-      <c r="B51" s="32" t="s">
-        <v>301</v>
-      </c>
-      <c r="C51" s="32" t="s">
-        <v>308</v>
-      </c>
-      <c r="D51" s="34" t="s">
+      <c r="D51" s="35" t="s">
         <v>72</v>
       </c>
-      <c r="E51" s="34" t="s">
+      <c r="E51" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F51" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="G51" s="48" t="str">
+      <c r="F51" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H51" s="48" t="str">
+      <c r="H51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="31" t="s">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="32" t="s">
+        <v>308</v>
+      </c>
+      <c r="B52" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="C52" s="33" t="s">
         <v>309</v>
       </c>
-      <c r="B52" s="32" t="s">
-        <v>301</v>
-      </c>
-      <c r="C52" s="32" t="s">
-        <v>310</v>
-      </c>
-      <c r="D52" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E52" s="34" t="s">
+      <c r="D52" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E52" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F52" s="34"/>
-      <c r="G52" s="48" t="str">
+      <c r="F52" s="35"/>
+      <c r="G52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E52,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Done</v>
       </c>
-      <c r="H52" s="48" t="str">
+      <c r="H52" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E52,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="31" t="s">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="32" t="s">
+        <v>310</v>
+      </c>
+      <c r="B53" s="33" t="s">
+        <v>300</v>
+      </c>
+      <c r="C53" s="33" t="s">
         <v>311</v>
       </c>
-      <c r="B53" s="32" t="s">
-        <v>301</v>
-      </c>
-      <c r="C53" s="32" t="s">
-        <v>312</v>
-      </c>
-      <c r="D53" s="34" t="s">
-        <v>213</v>
-      </c>
-      <c r="E53" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="F53" s="34"/>
-      <c r="G53" s="48" t="str">
+      <c r="D53" s="35" t="s">
+        <v>212</v>
+      </c>
+      <c r="E53" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="F53" s="35"/>
+      <c r="G53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H53" s="48" t="str">
+      <c r="H53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="31" t="s">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="32" t="s">
+        <v>312</v>
+      </c>
+      <c r="B54" s="33" t="s">
+        <v>284</v>
+      </c>
+      <c r="C54" s="33" t="s">
         <v>313</v>
       </c>
-      <c r="B54" s="32" t="s">
-        <v>285</v>
-      </c>
-      <c r="C54" s="32" t="s">
-        <v>314</v>
-      </c>
-      <c r="D54" s="34" t="s">
-        <v>161</v>
-      </c>
-      <c r="E54" s="34" t="s">
-        <v>182</v>
-      </c>
-      <c r="F54" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="G54" s="48" t="str">
+      <c r="D54" s="35" t="s">
+        <v>160</v>
+      </c>
+      <c r="E54" s="35" t="s">
+        <v>181</v>
+      </c>
+      <c r="F54" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="G54" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Not started</v>
       </c>
-      <c r="H54" s="48" t="str">
+      <c r="H54" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
@@ -5117,21 +5110,21 @@
   </sheetData>
   <autoFilter ref="A4:H54"/>
   <conditionalFormatting sqref="G5:G54">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D54">
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Must"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5154,368 +5147,368 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="31" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="B4" s="31" t="s">
         <v>317</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="C4" s="31" t="s">
         <v>318</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="D4" s="31" t="s">
         <v>319</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="E4" s="31" t="s">
         <v>320</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="F4" s="31" t="s">
         <v>321</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="G4" s="31" t="s">
         <v>322</v>
       </c>
-      <c r="G4" s="30" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="32" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="B5" s="35" t="s">
         <v>324</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="C5" s="50" t="s">
         <v>325</v>
       </c>
-      <c r="C5" s="49" t="s">
+      <c r="D5" s="33" t="s">
         <v>326</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="E5" s="33" t="s">
         <v>327</v>
       </c>
-      <c r="E5" s="32" t="s">
+      <c r="F5" s="33" t="s">
         <v>328</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="G5" s="35" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="32" t="s">
         <v>329</v>
       </c>
-      <c r="G5" s="34" t="s">
+      <c r="B6" s="35" t="s">
+        <v>330</v>
+      </c>
+      <c r="C6" s="50" t="s">
+        <v>331</v>
+      </c>
+      <c r="D6" s="33" t="s">
+        <v>332</v>
+      </c>
+      <c r="E6" s="33" t="s">
+        <v>333</v>
+      </c>
+      <c r="F6" s="33" t="s">
+        <v>334</v>
+      </c>
+      <c r="G6" s="35" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="32" t="s">
+        <v>335</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>336</v>
+      </c>
+      <c r="C7" s="50" t="s">
+        <v>337</v>
+      </c>
+      <c r="D7" s="33" t="s">
+        <v>338</v>
+      </c>
+      <c r="E7" s="33" t="s">
+        <v>339</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>340</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="32" t="s">
+        <v>341</v>
+      </c>
+      <c r="B8" s="35" t="s">
+        <v>342</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>343</v>
+      </c>
+      <c r="D8" s="33" t="s">
+        <v>344</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>345</v>
+      </c>
+      <c r="F8" s="33" t="s">
+        <v>346</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="32" t="s">
+        <v>347</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>348</v>
+      </c>
+      <c r="C9" s="50" t="s">
+        <v>349</v>
+      </c>
+      <c r="D9" s="33" t="s">
+        <v>350</v>
+      </c>
+      <c r="E9" s="33" t="s">
+        <v>351</v>
+      </c>
+      <c r="F9" s="33" t="s">
+        <v>352</v>
+      </c>
+      <c r="G9" s="35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="32" t="s">
+        <v>353</v>
+      </c>
+      <c r="B10" s="35" t="s">
+        <v>354</v>
+      </c>
+      <c r="C10" s="50" t="s">
+        <v>355</v>
+      </c>
+      <c r="D10" s="33" t="s">
+        <v>356</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>357</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>358</v>
+      </c>
+      <c r="G10" s="35" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="s">
-        <v>330</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>331</v>
-      </c>
-      <c r="C6" s="49" t="s">
-        <v>332</v>
-      </c>
-      <c r="D6" s="32" t="s">
-        <v>333</v>
-      </c>
-      <c r="E6" s="32" t="s">
-        <v>334</v>
-      </c>
-      <c r="F6" s="32" t="s">
-        <v>335</v>
-      </c>
-      <c r="G6" s="34" t="s">
+    <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="32" t="s">
+        <v>359</v>
+      </c>
+      <c r="B11" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>360</v>
+      </c>
+      <c r="D11" s="33" t="s">
+        <v>361</v>
+      </c>
+      <c r="E11" s="33" t="s">
+        <v>362</v>
+      </c>
+      <c r="F11" s="33" t="s">
+        <v>363</v>
+      </c>
+      <c r="G11" s="35" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
+        <v>364</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>365</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>366</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>367</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>368</v>
+      </c>
+      <c r="F12" s="33" t="s">
+        <v>369</v>
+      </c>
+      <c r="G12" s="35" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="s">
-        <v>336</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>337</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>338</v>
-      </c>
-      <c r="D7" s="32" t="s">
-        <v>339</v>
-      </c>
-      <c r="E7" s="32" t="s">
-        <v>340</v>
-      </c>
-      <c r="F7" s="32" t="s">
-        <v>341</v>
-      </c>
-      <c r="G7" s="34" t="s">
+    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="32" t="s">
+        <v>370</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>371</v>
+      </c>
+      <c r="C13" s="50" t="s">
+        <v>372</v>
+      </c>
+      <c r="D13" s="33" t="s">
+        <v>373</v>
+      </c>
+      <c r="E13" s="33" t="s">
+        <v>374</v>
+      </c>
+      <c r="F13" s="33" t="s">
+        <v>375</v>
+      </c>
+      <c r="G13" s="35" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
+        <v>376</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>377</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>378</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>379</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>380</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>381</v>
+      </c>
+      <c r="G14" s="35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>382</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>383</v>
+      </c>
+      <c r="C15" s="50" t="s">
+        <v>384</v>
+      </c>
+      <c r="D15" s="33" t="s">
+        <v>385</v>
+      </c>
+      <c r="E15" s="33" t="s">
+        <v>386</v>
+      </c>
+      <c r="F15" s="33" t="s">
+        <v>387</v>
+      </c>
+      <c r="G15" s="35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>388</v>
+      </c>
+      <c r="B16" s="35" t="s">
+        <v>389</v>
+      </c>
+      <c r="C16" s="50" t="s">
+        <v>390</v>
+      </c>
+      <c r="D16" s="33" t="s">
+        <v>391</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>392</v>
+      </c>
+      <c r="F16" s="33" t="s">
+        <v>393</v>
+      </c>
+      <c r="G16" s="35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>394</v>
+      </c>
+      <c r="B17" s="35" t="s">
+        <v>395</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>396</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>397</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>398</v>
+      </c>
+      <c r="F17" s="33" t="s">
+        <v>399</v>
+      </c>
+      <c r="G17" s="35" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="31" t="s">
-        <v>342</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>343</v>
-      </c>
-      <c r="C8" s="49" t="s">
-        <v>344</v>
-      </c>
-      <c r="D8" s="32" t="s">
-        <v>345</v>
-      </c>
-      <c r="E8" s="32" t="s">
-        <v>346</v>
-      </c>
-      <c r="F8" s="32" t="s">
-        <v>347</v>
-      </c>
-      <c r="G8" s="34" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="31" t="s">
-        <v>348</v>
-      </c>
-      <c r="B9" s="34" t="s">
-        <v>349</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>350</v>
-      </c>
-      <c r="D9" s="32" t="s">
-        <v>351</v>
-      </c>
-      <c r="E9" s="32" t="s">
-        <v>352</v>
-      </c>
-      <c r="F9" s="32" t="s">
-        <v>353</v>
-      </c>
-      <c r="G9" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="31" t="s">
-        <v>354</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>355</v>
-      </c>
-      <c r="C10" s="49" t="s">
-        <v>356</v>
-      </c>
-      <c r="D10" s="32" t="s">
-        <v>357</v>
-      </c>
-      <c r="E10" s="32" t="s">
-        <v>358</v>
-      </c>
-      <c r="F10" s="32" t="s">
-        <v>359</v>
-      </c>
-      <c r="G10" s="34" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="31" t="s">
-        <v>360</v>
-      </c>
-      <c r="B11" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="49" t="s">
-        <v>361</v>
-      </c>
-      <c r="D11" s="32" t="s">
-        <v>362</v>
-      </c>
-      <c r="E11" s="32" t="s">
-        <v>363</v>
-      </c>
-      <c r="F11" s="32" t="s">
-        <v>364</v>
-      </c>
-      <c r="G11" s="34" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="31" t="s">
-        <v>365</v>
-      </c>
-      <c r="B12" s="34" t="s">
-        <v>366</v>
-      </c>
-      <c r="C12" s="49" t="s">
-        <v>367</v>
-      </c>
-      <c r="D12" s="32" t="s">
-        <v>368</v>
-      </c>
-      <c r="E12" s="32" t="s">
-        <v>369</v>
-      </c>
-      <c r="F12" s="32" t="s">
-        <v>370</v>
-      </c>
-      <c r="G12" s="34" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="31" t="s">
-        <v>371</v>
-      </c>
-      <c r="B13" s="34" t="s">
-        <v>372</v>
-      </c>
-      <c r="C13" s="49" t="s">
-        <v>373</v>
-      </c>
-      <c r="D13" s="32" t="s">
-        <v>374</v>
-      </c>
-      <c r="E13" s="32" t="s">
-        <v>375</v>
-      </c>
-      <c r="F13" s="32" t="s">
-        <v>376</v>
-      </c>
-      <c r="G13" s="34" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
-        <v>377</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>378</v>
-      </c>
-      <c r="C14" s="49" t="s">
-        <v>379</v>
-      </c>
-      <c r="D14" s="32" t="s">
-        <v>380</v>
-      </c>
-      <c r="E14" s="32" t="s">
-        <v>381</v>
-      </c>
-      <c r="F14" s="32" t="s">
-        <v>382</v>
-      </c>
-      <c r="G14" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>383</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>384</v>
-      </c>
-      <c r="C15" s="49" t="s">
-        <v>385</v>
-      </c>
-      <c r="D15" s="32" t="s">
-        <v>386</v>
-      </c>
-      <c r="E15" s="32" t="s">
-        <v>387</v>
-      </c>
-      <c r="F15" s="32" t="s">
-        <v>388</v>
-      </c>
-      <c r="G15" s="34" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
-        <v>389</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>390</v>
-      </c>
-      <c r="C16" s="49" t="s">
-        <v>391</v>
-      </c>
-      <c r="D16" s="32" t="s">
-        <v>392</v>
-      </c>
-      <c r="E16" s="32" t="s">
-        <v>393</v>
-      </c>
-      <c r="F16" s="32" t="s">
-        <v>394</v>
-      </c>
-      <c r="G16" s="34" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
-        <v>395</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>396</v>
-      </c>
-      <c r="C17" s="49" t="s">
-        <v>397</v>
-      </c>
-      <c r="D17" s="32" t="s">
-        <v>398</v>
-      </c>
-      <c r="E17" s="32" t="s">
-        <v>399</v>
-      </c>
-      <c r="F17" s="32" t="s">
+    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="32" t="s">
         <v>400</v>
       </c>
-      <c r="G17" s="34" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="31" t="s">
+      <c r="B18" s="35" t="s">
         <v>401</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="C18" s="50" t="s">
         <v>402</v>
       </c>
-      <c r="C18" s="49" t="s">
+      <c r="D18" s="33" t="s">
         <v>403</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="E18" s="33" t="s">
         <v>404</v>
       </c>
-      <c r="E18" s="32" t="s">
+      <c r="F18" s="33" t="s">
         <v>405</v>
       </c>
-      <c r="F18" s="32" t="s">
-        <v>406</v>
-      </c>
-      <c r="G18" s="34" t="s">
-        <v>182</v>
+      <c r="G18" s="35" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-08 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="407">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -517,7 +517,7 @@
     <t xml:space="preserve">Why citations rendered from structured data; streaming UX; accessibility basics; per-business route from day one, so PR-15 needs no rework</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #10. Chat API takes the business slug (/b/[slug]). One review round: bounded business cache, history race, reload mid-answer polling, memoized streaming, repeated save_lead deduped in the loop.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-09</t>
@@ -551,6 +551,9 @@
   </si>
   <si>
     <t xml:space="preserve">PR-06, PR-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-10</t>
@@ -2396,7 +2399,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2432,7 +2435,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,7 +2444,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.372881355932203</v>
+        <v>0.474576271186441</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2459,7 +2462,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2683,7 +2686,7 @@
       </c>
       <c r="D30" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A30,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3287,13 +3290,15 @@
         <v>20</v>
       </c>
       <c r="M12" s="37" t="s">
-        <v>134</v>
+        <v>29</v>
       </c>
       <c r="N12" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A12)</f>
         <v>6</v>
       </c>
-      <c r="O12" s="38"/>
+      <c r="O12" s="38" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
@@ -3333,7 +3338,7 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
@@ -3343,13 +3348,13 @@
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D14" s="43" t="s">
         <v>35</v>
@@ -3358,16 +3363,16 @@
         <v>72</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G14" s="33" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H14" s="33" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J14" s="35" t="s">
         <v>95</v>
@@ -3379,7 +3384,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3389,13 +3394,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3404,16 +3409,16 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J15" s="35" t="s">
         <v>111</v>
@@ -3425,7 +3430,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3435,31 +3440,31 @@
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>119</v>
@@ -3471,7 +3476,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3481,13 +3486,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3496,19 +3501,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3517,7 +3522,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3527,13 +3532,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3542,19 +3547,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3563,7 +3568,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3573,34 +3578,34 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3609,19 +3614,19 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3646,7 +3651,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3723,49 +3728,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3778,7 +3783,7 @@
       </c>
       <c r="G5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H5" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3787,13 +3792,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3806,7 +3811,7 @@
       </c>
       <c r="G6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H6" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3815,13 +3820,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3834,7 +3839,7 @@
       </c>
       <c r="G7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H7" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3843,13 +3848,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3860,7 +3865,7 @@
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H8" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3869,16 +3874,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3886,7 +3891,7 @@
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H9" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3895,13 +3900,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3921,13 +3926,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3947,13 +3952,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3973,13 +3978,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4001,13 +4006,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4027,13 +4032,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4053,13 +4058,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4081,13 +4086,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4109,13 +4114,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4137,13 +4142,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4163,13 +4168,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4191,13 +4196,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4217,13 +4222,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4245,13 +4250,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4273,13 +4278,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4299,13 +4304,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4327,13 +4332,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4353,13 +4358,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4381,13 +4386,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4409,13 +4414,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4437,19 +4442,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E30" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F30" s="35" t="s">
         <v>95</v>
@@ -4465,13 +4470,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4480,7 +4485,7 @@
         <v>95</v>
       </c>
       <c r="F31" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G31" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E31,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4493,19 +4498,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E32" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
@@ -4519,19 +4524,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E33" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
@@ -4545,19 +4550,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E34" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F34" s="35" t="s">
         <v>103</v>
@@ -4573,19 +4578,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4599,19 +4604,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4625,19 +4630,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4651,19 +4656,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4677,19 +4682,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F39" s="35" t="s">
         <v>111</v>
@@ -4705,19 +4710,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4731,22 +4736,22 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F41" s="35" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4759,13 +4764,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4774,7 +4779,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4787,13 +4792,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4813,13 +4818,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4828,7 +4833,7 @@
         <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4841,13 +4846,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4867,13 +4872,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4893,13 +4898,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4908,11 +4913,11 @@
         <v>127</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4921,13 +4926,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4949,13 +4954,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4975,13 +4980,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5001,13 +5006,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5016,7 +5021,7 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5029,16 +5034,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E52" s="35" t="s">
         <v>111</v>
@@ -5055,19 +5060,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5081,22 +5086,22 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D54" s="35" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F54" s="35" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G54" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5158,55 +5163,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5214,22 +5219,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5237,22 +5242,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5260,22 +5265,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5283,22 +5288,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5306,22 +5311,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5329,22 +5334,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5352,22 +5357,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5375,22 +5380,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5398,22 +5403,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5421,22 +5426,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5444,22 +5449,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5467,22 +5472,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5490,25 +5495,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add realtime voice over WebRTC
Voice mode for the customer chat, on the OpenAI Realtime API. Audio goes
browser <-> OpenAI; the server opens the call for the browser's SDP offer
(no key or token in the browser), runs the tools the model calls through
the same executor as text chat, and stores transcripts as voice messages
in the same conversation, in conversation order.

A voice answer's citations and action cards are copied from the tool
calls the server ran since the previous answer (new tool_calls.sources
column), never taken from the browser.

Fixes turn_in_progress to count only text questions: voice questions
blocked typing for 60 s after a call (found in live testing).

UI: permission explainer, voice panel with a level-following orb, states,
mute/end, blocked-microphone and disconnected states, live captions in
the thread.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -532,10 +532,10 @@
     <t xml:space="preserve">US-2.1, US-2.2, US-2.3, US-2.4, US-2.5, US-2.6, US-6.4, US-12.1</t>
   </si>
   <si>
-    <t xml:space="preserve">- POST /api/realtime/session: mint ephemeral token with same instructions + tool definitions + recent history
+    <t xml:space="preserve">- POST /api/voice/session: the server opens the Realtime call for the browser's SDP offer, with the same instructions + tool definitions + recent history (no key or token in the browser)
 - Browser WebRTC: mic track, remote audio, data channel
 - Server VAD (natural turn-taking, barge-in)
-- Tool relay: data channel function_call -&gt; POST /api/tools -&gt; function_call_output
+- Tool relay: data channel function_call -&gt; POST /api/voice/tool -&gt; function_call_output
 - Persist user/assistant transcripts (channel=voice)
 - Voice panel UI: states, orb, mute, end, permission &amp; error handling</t>
   </si>
@@ -1236,7 +1236,7 @@
     <t xml:space="preserve">D-07</t>
   </si>
   <si>
-    <t xml:space="preserve">OpenAI Realtime over WebRTC with ephemeral tokens</t>
+    <t xml:space="preserve">OpenAI Realtime over WebRTC; the server opens the call (relays the SDP offer), so no key or token reaches the browser</t>
   </si>
   <si>
     <t xml:space="preserve">Whisper STT + LLM + TTS pipeline</t>
@@ -1245,7 +1245,7 @@
     <t xml:space="preserve">Lowest latency, natural turn-taking and barge-in; key never in browser</t>
   </si>
   <si>
-    <t xml:space="preserve">Higher cost per minute; tool calls relayed via browser</t>
+    <t xml:space="preserve">Higher cost per minute; tool calls and transcripts are relayed by the browser (a server-side connection to the call is the production next step)</t>
   </si>
   <si>
     <t xml:space="preserve">D-08</t>

</xml_diff>

<commit_message>
Mark PR-09 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="408">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -553,7 +553,7 @@
     <t xml:space="preserve">PR-06, PR-07</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #11. Server opens the call (no key or token in the browser); per-call secret on tool/transcript requests; cards attached by tool-call id; interruptions keep what was heard. Live-tested with synthetic speech. Rate limit + call cap moved to PR-13.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-10</t>
@@ -581,6 +581,9 @@
   </si>
   <si>
     <t xml:space="preserve">Synchronous vs background ingestion (and when to move to a queue); admin auth out of scope and how you'd add it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-11</t>
@@ -2399,7 +2402,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2435,7 +2438,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2444,7 +2447,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.474576271186441</v>
+        <v>0.610169491525424</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2462,7 +2465,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2703,7 +2706,7 @@
       </c>
       <c r="D31" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A31,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3338,13 +3341,15 @@
         <v>20</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>143</v>
+        <v>29</v>
       </c>
       <c r="N13" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A13)</f>
         <v>8</v>
       </c>
-      <c r="O13" s="38"/>
+      <c r="O13" s="38" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
@@ -3384,7 +3389,7 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
@@ -3394,13 +3399,13 @@
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D15" s="43" t="s">
         <v>35</v>
@@ -3409,16 +3414,16 @@
         <v>72</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J15" s="35" t="s">
         <v>111</v>
@@ -3430,7 +3435,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3440,31 +3445,31 @@
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>119</v>
@@ -3476,7 +3481,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3486,13 +3491,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3501,19 +3506,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3522,7 +3527,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3532,13 +3537,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3547,19 +3552,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3568,7 +3573,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3578,34 +3583,34 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3614,19 +3619,19 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3651,7 +3656,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3728,49 +3733,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3792,13 +3797,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3820,13 +3825,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3848,13 +3853,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3874,16 +3879,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3900,13 +3905,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3917,7 +3922,7 @@
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H10" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3926,13 +3931,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3943,7 +3948,7 @@
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H11" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3952,13 +3957,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3969,7 +3974,7 @@
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H12" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -3978,13 +3983,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -3997,7 +4002,7 @@
       </c>
       <c r="G13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H13" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4006,13 +4011,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4023,7 +4028,7 @@
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H14" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4032,13 +4037,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4049,7 +4054,7 @@
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H15" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4058,13 +4063,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4086,13 +4091,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4114,13 +4119,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4142,13 +4147,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4168,13 +4173,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4196,13 +4201,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4222,13 +4227,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4250,13 +4255,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4278,13 +4283,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4304,13 +4309,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4332,13 +4337,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4358,13 +4363,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4386,13 +4391,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4414,13 +4419,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4433,7 +4438,7 @@
       </c>
       <c r="G29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H29" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4442,13 +4447,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4470,13 +4475,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4498,13 +4503,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4524,16 +4529,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
@@ -4550,16 +4555,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4578,19 +4583,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E35" s="35" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
@@ -4604,19 +4609,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
       </c>
       <c r="E36" s="35" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
@@ -4630,19 +4635,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E37" s="35" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
@@ -4656,19 +4661,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4682,19 +4687,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F39" s="35" t="s">
         <v>111</v>
@@ -4710,19 +4715,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4736,22 +4741,22 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F41" s="35" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4764,13 +4769,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4779,7 +4784,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4792,13 +4797,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4818,13 +4823,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4833,7 +4838,7 @@
         <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4846,13 +4851,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4872,13 +4877,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4898,13 +4903,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4913,7 +4918,7 @@
         <v>127</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4926,13 +4931,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4945,7 +4950,7 @@
       </c>
       <c r="G48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H48" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4954,13 +4959,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4980,13 +4985,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5006,13 +5011,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5021,7 +5026,7 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5034,16 +5039,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E52" s="35" t="s">
         <v>111</v>
@@ -5060,19 +5065,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5086,19 +5091,19 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D54" s="35" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F54" s="35" t="s">
         <v>144</v>
@@ -5163,55 +5168,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5219,22 +5224,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5242,22 +5247,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5265,22 +5270,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5288,22 +5293,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5311,22 +5316,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5334,22 +5339,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5357,22 +5362,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5380,22 +5385,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5403,22 +5408,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5426,22 +5431,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5449,22 +5454,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5472,22 +5477,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5495,25 +5500,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-10 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="409">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -583,7 +583,7 @@
     <t xml:space="preserve">Synchronous vs background ingestion (and when to move to a queue); admin auth out of scope and how you'd add it</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #12. Admin URLs carry the business (/admin/[slug]). Synchronous ingestion via the existing pipeline. Review round: capped upload body, test search = assistant's search, Replace for same-title uploads, interrupted uploads, plain error messages.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-11</t>
@@ -609,6 +609,9 @@
   </si>
   <si>
     <t xml:space="preserve">Pagination/limits on lists; timezone handling (store UTC, display business tz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-12</t>
@@ -2403,7 +2406,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2439,7 +2442,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2448,7 +2451,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.610169491525424</v>
+        <v>0.677966101694915</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2466,7 +2469,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2724,7 +2727,7 @@
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3390,13 +3393,15 @@
         <v>20</v>
       </c>
       <c r="M14" s="37" t="s">
-        <v>151</v>
+        <v>29</v>
       </c>
       <c r="N14" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A14)</f>
         <v>4</v>
       </c>
-      <c r="O14" s="38"/>
+      <c r="O14" s="38" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
@@ -3436,7 +3441,7 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
@@ -3446,31 +3451,31 @@
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D16" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G16" s="33" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H16" s="33" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I16" s="33" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="J16" s="35" t="s">
         <v>119</v>
@@ -3482,7 +3487,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3492,13 +3497,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3507,19 +3512,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3528,7 +3533,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3538,13 +3543,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3553,19 +3558,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3574,7 +3579,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3584,34 +3589,34 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
       </c>
       <c r="E19" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3620,19 +3625,19 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3657,7 +3662,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -3734,49 +3739,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3798,13 +3803,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3826,13 +3831,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3854,13 +3859,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3880,16 +3885,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3906,13 +3911,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3932,13 +3937,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3958,13 +3963,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3984,13 +3989,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4012,13 +4017,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4038,13 +4043,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4064,13 +4069,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4092,13 +4097,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4120,13 +4125,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4148,13 +4153,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4174,13 +4179,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4202,13 +4207,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4228,13 +4233,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4256,13 +4261,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4284,13 +4289,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4310,13 +4315,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4338,13 +4343,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4364,13 +4369,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4392,13 +4397,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4420,13 +4425,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4448,13 +4453,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4467,7 +4472,7 @@
       </c>
       <c r="G30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H30" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4476,13 +4481,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4504,13 +4509,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4521,7 +4526,7 @@
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H32" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4530,16 +4535,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
@@ -4547,7 +4552,7 @@
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H33" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4556,16 +4561,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4575,7 +4580,7 @@
       </c>
       <c r="G34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H34" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4584,13 +4589,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
@@ -4610,13 +4615,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
@@ -4636,16 +4641,16 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E37" s="35" t="s">
         <v>152</v>
@@ -4662,19 +4667,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D38" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E38" s="35" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
@@ -4688,19 +4693,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E39" s="35" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F39" s="35" t="s">
         <v>111</v>
@@ -4716,19 +4721,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
@@ -4742,22 +4747,22 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F41" s="35" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4770,13 +4775,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4785,7 +4790,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4798,13 +4803,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4824,13 +4829,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4839,7 +4844,7 @@
         <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4852,13 +4857,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4878,13 +4883,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4904,13 +4909,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4919,7 +4924,7 @@
         <v>127</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4932,13 +4937,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4960,13 +4965,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4986,13 +4991,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5012,13 +5017,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5027,7 +5032,7 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5040,16 +5045,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D52" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E52" s="35" t="s">
         <v>111</v>
@@ -5066,19 +5071,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5092,19 +5097,19 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D54" s="35" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F54" s="35" t="s">
         <v>144</v>
@@ -5169,55 +5174,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5225,22 +5230,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5248,22 +5253,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5271,22 +5276,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5294,22 +5299,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5317,22 +5322,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5340,22 +5345,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5363,22 +5368,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5386,22 +5391,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5409,22 +5414,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5432,22 +5437,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5455,22 +5460,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5478,22 +5483,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5501,25 +5506,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-11 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="410">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -611,7 +611,7 @@
     <t xml:space="preserve">Pagination/limits on lists; timezone handling (store UTC, display business tz)</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #13. Overview, leads (search, drawer), consultations (upcoming first, optimistic status change). Times in the business timezone with per-row zone labels. Admin sign-in was built then removed on request: the admin stays public (A1, 'Demo mode · no login').</t>
   </si>
   <si>
     <t xml:space="preserve">PR-12</t>
@@ -638,6 +638,9 @@
   </si>
   <si>
     <t xml:space="preserve">Observability of agent actions; knowledge-gap loop as product value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-13</t>
@@ -2406,7 +2409,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2442,7 +2445,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>20</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2451,7 +2454,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.677966101694915</v>
+        <v>0.728813559322034</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2469,7 +2472,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">COUNTIFS('Story Coverage'!$D:$D,"Must",'Story Coverage'!$G:$G,"Done")</f>
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2727,7 +2730,7 @@
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3441,13 +3444,15 @@
         <v>21</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>159</v>
+        <v>29</v>
       </c>
       <c r="N15" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A15)</f>
         <v>3</v>
       </c>
-      <c r="O15" s="38"/>
+      <c r="O15" s="38" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
@@ -3487,7 +3492,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
@@ -3497,13 +3502,13 @@
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>36</v>
@@ -3512,19 +3517,19 @@
         <v>72</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G17" s="33" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I17" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J17" s="35" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K17" s="36" t="n">
         <v>1.5</v>
@@ -3533,7 +3538,7 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
@@ -3543,13 +3548,13 @@
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3558,19 +3563,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3579,7 +3584,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3589,13 +3594,13 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
@@ -3604,19 +3609,19 @@
         <v>163</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3625,19 +3630,19 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3662,7 +3667,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3739,49 +3744,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3803,13 +3808,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3831,13 +3836,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3859,13 +3864,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3885,16 +3890,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3911,13 +3916,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3937,13 +3942,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3963,13 +3968,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3989,13 +3994,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4017,13 +4022,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4043,13 +4048,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4069,13 +4074,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4097,13 +4102,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4125,13 +4130,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4153,13 +4158,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4179,13 +4184,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4207,13 +4212,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4233,13 +4238,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4261,13 +4266,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4289,13 +4294,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4315,13 +4320,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4343,13 +4348,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4369,13 +4374,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4397,13 +4402,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4425,13 +4430,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4453,13 +4458,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4481,13 +4486,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4509,13 +4514,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4535,16 +4540,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
@@ -4561,16 +4566,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4589,13 +4594,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
@@ -4606,7 +4611,7 @@
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H35" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4615,13 +4620,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
@@ -4632,7 +4637,7 @@
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H36" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4641,13 +4646,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D37" s="35" t="s">
         <v>163</v>
@@ -4658,7 +4663,7 @@
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H37" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4667,13 +4672,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D38" s="35" t="s">
         <v>163</v>
@@ -4693,13 +4698,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D39" s="35" t="s">
         <v>163</v>
@@ -4721,16 +4726,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E40" s="35" t="s">
         <v>160</v>
@@ -4747,19 +4752,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D41" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F41" s="35" t="s">
         <v>160</v>
@@ -4775,13 +4780,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4790,7 +4795,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G42" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4803,13 +4808,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4829,13 +4834,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4844,7 +4849,7 @@
         <v>119</v>
       </c>
       <c r="F44" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G44" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4857,13 +4862,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4883,13 +4888,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4909,13 +4914,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4924,7 +4929,7 @@
         <v>127</v>
       </c>
       <c r="F47" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G47" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4937,13 +4942,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4965,13 +4970,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4991,13 +4996,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5017,13 +5022,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5032,7 +5037,7 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G51" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5045,13 +5050,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D52" s="35" t="s">
         <v>163</v>
@@ -5071,19 +5076,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E53" s="35" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
@@ -5097,19 +5102,19 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D54" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F54" s="35" t="s">
         <v>144</v>
@@ -5174,55 +5179,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5230,22 +5235,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5253,22 +5258,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5276,22 +5281,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5299,22 +5304,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5322,22 +5327,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5345,22 +5350,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5368,22 +5373,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5391,22 +5396,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5414,22 +5419,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5437,22 +5442,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5460,22 +5465,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5483,22 +5488,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5506,25 +5511,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-13 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="411">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -672,6 +672,9 @@
   </si>
   <si>
     <t xml:space="preserve">PR-07, PR-08, PR-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merged: PR #14. Postgres rate limits in tiers (visitor, then business ceiling; per-IP via TRUSTED_IP_HEADER), SIMULATE_DB_FAILURE, voice call cap with server hang-up, structured tool logs, prompt fixes from live probes (off-topic, yes/no conditions, over-refusal). README failure-test checklist.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-14</t>
@@ -2409,7 +2412,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2445,7 +2448,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>21.5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2454,7 +2457,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.728813559322034</v>
+        <v>0.779661016949153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2747,7 +2750,7 @@
       </c>
       <c r="D33" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A33,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3538,23 +3541,25 @@
         <v>21</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>168</v>
+        <v>29</v>
       </c>
       <c r="N17" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A17)</f>
         <v>1</v>
       </c>
-      <c r="O17" s="38"/>
+      <c r="O17" s="38" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D18" s="45" t="s">
         <v>37</v>
@@ -3563,19 +3568,19 @@
         <v>72</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G18" s="33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H18" s="33" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I18" s="33" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J18" s="35" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K18" s="36" t="n">
         <v>2</v>
@@ -3594,13 +3599,13 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
@@ -3609,19 +3614,19 @@
         <v>163</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3637,12 +3642,12 @@
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3667,7 +3672,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -3744,49 +3749,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3808,13 +3813,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3836,13 +3841,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3864,13 +3869,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3890,16 +3895,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3916,13 +3921,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3942,13 +3947,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3968,13 +3973,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3994,13 +3999,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4022,13 +4027,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4048,13 +4053,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4074,13 +4079,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4102,13 +4107,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4130,13 +4135,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4158,13 +4163,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4184,13 +4189,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4212,13 +4217,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4238,13 +4243,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4266,13 +4271,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4294,13 +4299,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4320,13 +4325,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4348,13 +4353,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4374,13 +4379,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4402,13 +4407,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4430,13 +4435,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4458,13 +4463,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4486,13 +4491,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4514,13 +4519,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4540,16 +4545,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
@@ -4566,16 +4571,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4594,13 +4599,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
@@ -4620,13 +4625,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
@@ -4646,13 +4651,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D37" s="35" t="s">
         <v>163</v>
@@ -4672,13 +4677,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D38" s="35" t="s">
         <v>163</v>
@@ -4698,13 +4703,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D39" s="35" t="s">
         <v>163</v>
@@ -4726,16 +4731,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E40" s="35" t="s">
         <v>160</v>
@@ -4752,19 +4757,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D41" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F41" s="35" t="s">
         <v>160</v>
@@ -4780,13 +4785,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4808,13 +4813,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4834,13 +4839,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4862,13 +4867,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4888,13 +4893,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4914,13 +4919,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4942,13 +4947,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4970,13 +4975,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4996,13 +5001,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5022,13 +5027,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5050,13 +5055,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D52" s="35" t="s">
         <v>163</v>
@@ -5076,16 +5081,16 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E53" s="35" t="s">
         <v>169</v>
@@ -5093,7 +5098,7 @@
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H53" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5102,19 +5107,19 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D54" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F54" s="35" t="s">
         <v>144</v>
@@ -5179,55 +5184,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5235,22 +5240,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5258,22 +5263,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5281,22 +5286,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5304,22 +5309,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5327,22 +5332,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5350,22 +5355,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5373,22 +5378,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5396,22 +5401,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5419,22 +5424,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5442,22 +5447,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5465,22 +5470,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5488,22 +5493,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5511,25 +5516,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-12 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="412">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -640,7 +640,7 @@
     <t xml:space="preserve">Observability of agent actions; knowledge-gap loop as product value</t>
   </si>
   <si>
-    <t xml:space="preserve">Not started</t>
+    <t xml:space="preserve">Merged: PR #15. Conversations list + transcript with inline tool-call rows (args/result JSON, duration, failures red and open); voice tool calls placed by their link to the answer, text by time. Overview: questions the assistant couldn't answer (search found:false), linked to the conversation. Lead drawer links to the conversation.</t>
   </si>
   <si>
     <t xml:space="preserve">PR-13</t>
@@ -702,6 +702,9 @@
   </si>
   <si>
     <t xml:space="preserve">All</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not started</t>
   </si>
   <si>
     <t xml:space="preserve">PR-15</t>
@@ -2412,7 +2415,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2448,7 +2451,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>23</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2457,7 +2460,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.779661016949153</v>
+        <v>0.830508474576271</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2733,7 +2736,7 @@
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3495,13 +3498,15 @@
         <v>22</v>
       </c>
       <c r="M16" s="37" t="s">
-        <v>168</v>
+        <v>29</v>
       </c>
       <c r="N16" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A16)</f>
         <v>3</v>
       </c>
-      <c r="O16" s="38"/>
+      <c r="O16" s="38" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
@@ -3589,7 +3594,7 @@
         <v>21</v>
       </c>
       <c r="M18" s="37" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="N18" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A18)</f>
@@ -3599,13 +3604,13 @@
     </row>
     <row r="19" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D19" s="43" t="s">
         <v>35</v>
@@ -3614,19 +3619,19 @@
         <v>163</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G19" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J19" s="35" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K19" s="36" t="n">
         <v>3</v>
@@ -3635,19 +3640,19 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
         <v>2</v>
       </c>
       <c r="O19" s="38" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
@@ -3672,7 +3677,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K21" s="16" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3749,49 +3754,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3813,13 +3818,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3841,13 +3846,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3869,13 +3874,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3895,16 +3900,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
@@ -3921,13 +3926,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3947,13 +3952,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3973,13 +3978,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3999,13 +4004,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4027,13 +4032,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4053,13 +4058,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4079,13 +4084,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4107,13 +4112,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4135,13 +4140,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4163,13 +4168,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4189,13 +4194,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4217,13 +4222,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4243,13 +4248,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4271,13 +4276,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4299,13 +4304,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4325,13 +4330,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4353,13 +4358,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4379,13 +4384,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4407,13 +4412,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4435,13 +4440,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4463,13 +4468,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4491,13 +4496,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4519,13 +4524,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4545,16 +4550,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
@@ -4571,16 +4576,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4599,13 +4604,13 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
@@ -4625,13 +4630,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
@@ -4651,13 +4656,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D37" s="35" t="s">
         <v>163</v>
@@ -4677,13 +4682,13 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D38" s="35" t="s">
         <v>163</v>
@@ -4694,7 +4699,7 @@
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H38" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4703,13 +4708,13 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D39" s="35" t="s">
         <v>163</v>
@@ -4722,7 +4727,7 @@
       </c>
       <c r="G39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H39" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4731,16 +4736,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E40" s="35" t="s">
         <v>160</v>
@@ -4748,7 +4753,7 @@
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H40" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -4757,19 +4762,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D41" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E41" s="35" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F41" s="35" t="s">
         <v>160</v>
@@ -4785,13 +4790,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4813,13 +4818,13 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4839,13 +4844,13 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4867,13 +4872,13 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4893,13 +4898,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4919,13 +4924,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4947,13 +4952,13 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4975,13 +4980,13 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -5001,13 +5006,13 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5027,13 +5032,13 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5055,13 +5060,13 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D52" s="35" t="s">
         <v>163</v>
@@ -5081,16 +5086,16 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E53" s="35" t="s">
         <v>169</v>
@@ -5107,19 +5112,19 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D54" s="35" t="s">
         <v>163</v>
       </c>
       <c r="E54" s="35" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F54" s="35" t="s">
         <v>144</v>
@@ -5184,55 +5189,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5240,22 +5245,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5263,22 +5268,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5286,22 +5291,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5309,22 +5314,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5332,22 +5337,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5355,22 +5360,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5378,22 +5383,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5401,22 +5406,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5424,22 +5429,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5447,22 +5452,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5470,22 +5475,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5493,22 +5498,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5516,25 +5521,25 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G18" s="35" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark PR-15 done in the delivery plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -739,7 +739,7 @@
     <t xml:space="preserve">PR-08, PR-10</t>
   </si>
   <si>
-    <t xml:space="preserve">Agreed Oct 11. Core requirements first; this is the first item dropped if time runs short.</t>
+    <t xml:space="preserve">Merged: PR #17. Home page lists businesses; admin business switcher, New business and Settings (changes apply to the next message); assistant guidelines per business (clinic rules moved out of the shared prompt); sessions and rate limits keyed by business id so renames keep them; sample-gym data for the live demo.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B10" s="7" t="n">
         <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>24.5</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.830508474576271</v>
+        <v>0.932203389830508</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="D32" s="18" t="n">
         <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3640,7 +3640,7 @@
         <v>21</v>
       </c>
       <c r="M19" s="37" t="s">
-        <v>186</v>
+        <v>29</v>
       </c>
       <c r="N19" s="35" t="n">
         <f aca="false">COUNTIF('Story Coverage'!$E:$E,A19)</f>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="G41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H41" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="G54" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="H54" s="49" t="str">
         <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>

</xml_diff>

<commit_message>
Guards around the agent (PR-16)
- Input guard: a small model classifies every customer message
  (injection, authority claim, internals, off-topic), in parallel with
  the agent. Nothing is shown and no tool runs until it clears; a block
  stops the agent and sends a standard reply. Reads the business
  guidelines; learns from similar past blocks (same business).
- Output checks on every answer: canary (prompt leak), figures (every
  price, percentage, time, phone must be in this turn's evidence), scope
  (about the business). One rewrite, then a safe reply; the streamed
  bubble is replaced and only the replacement is saved.
- Voice: the same checks after the fact (flagged, not blocked).
- flags table; transcript marks; overview panel.
- npm run eval:guards: generated attacks, replayed blocks and generated
  normal questions, on a throwaway copy of the business.
- Plan: PR-16 row, decision D-15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-plan.xlsx
+++ b/docs/project-plan.xlsx
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="430">
   <si>
     <t xml:space="preserve">AI Customer Assistant - Delivery Plan</t>
   </si>
@@ -742,6 +742,42 @@
     <t xml:space="preserve">Merged: PR #17. Home page lists businesses; admin business switcher, New business and Settings (changes apply to the next message); assistant guidelines per business (clinic rules moved out of the shared prompt); sessions and rate limits keyed by business id so renames keep them; sample-gym data for the live demo.</t>
   </si>
   <si>
+    <t xml:space="preserve">PR-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feat/16-guards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guards around the agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-12.4, US-3.1, US-3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Input guard: small model classifies every message (injection, authority claim, internals, off-topic) in parallel with the agent; nothing shown and no tool run until it clears; reads the business guidelines; learns from past blocks (similar examples)
+- Output checks on every answer: canary (prompt leak), figures (every price/time/phone must be in this turn's evidence), scope (about the business); one rewrite, then a safe reply; streamed bubble replaced
+- Voice: same checks after the fact (flag, not block)
+- flags table; admin transcript marks and overview count
+- eval:guards: generated attacks + replayed blocks + generated normal questions, on a throwaway copy of the business</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- The founder-style message is blocked
+- An invented price never stays on screen
+- eval: attacks resisted up, normal questions wrongly blocked about 0%, added latency measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guarantees in code, prompt for style; platform rules vs business rules (admins can add, not remove); fail open; voice can't be unsaid; why generated evals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PR-12, PR-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measured on Lakeside: attacks resisted 19/25 without guards, 25/25 with (twice); normal questions wrongly blocked 0/20; p50 1.4-1.8 s.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
@@ -859,6 +895,9 @@
     <t xml:space="preserve">Accurate answers from the business's documents</t>
   </si>
   <si>
+    <t xml:space="preserve">PR-04, PR-16</t>
+  </si>
+  <si>
     <t xml:space="preserve">US-3.2</t>
   </si>
   <si>
@@ -1096,6 +1135,9 @@
     <t xml:space="preserve">Prompt-injection resistance</t>
   </si>
   <si>
+    <t xml:space="preserve">PR-13, PR-16</t>
+  </si>
+  <si>
     <t xml:space="preserve">US-12.5</t>
   </si>
   <si>
@@ -1388,6 +1430,24 @@
   </si>
   <si>
     <t xml:space="preserve">A picker isn't a real customer flow (customers arrive from the business's own website); tenant-scoped admin auth would be needed before any deployment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guarding the agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guards in code around every turn: input classifier (parallel, small model), canary, figure check against evidence, scope check; replace a failed answer; flags table the guard learns from; generated attack evals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More prompt rules; a moderation API only; a guard model on every token (blocking streams)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A prompt can be talked around (a 'founder' message got the assistant to list its rules). Code checks don't depend on the model obeying; numbers are the costliest mistake and are checkable exactly; the classifier runs in parallel so it costs ~no time; flags make it learn without code changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One small-model call per message plus one per answer; a rare flicker when an answer is replaced; voice can only be flagged after it is heard; generated evals vary per run</t>
   </si>
 </sst>
 </file>
@@ -2405,8 +2465,8 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTA('PR Plan'!$A$5:$A$19)</f>
-        <v>15</v>
+        <f aca="false">COUNTA('PR Plan'!$A$5:$A$20)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2414,7 +2474,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$20,"Done")</f>
         <v>14</v>
       </c>
     </row>
@@ -2423,8 +2483,8 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"In progress")+COUNTIF('PR Plan'!$M$5:$M$19,"In review")</f>
-        <v>0</v>
+        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$20,"In progress")+COUNTIF('PR Plan'!$M$5:$M$20,"In review")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2432,7 +2492,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$19,"Blocked")</f>
+        <f aca="false">COUNTIF('PR Plan'!$M$5:$M$20,"Blocked")</f>
         <v>0</v>
       </c>
     </row>
@@ -2441,8 +2501,8 @@
         <v>7</v>
       </c>
       <c r="B9" s="7" t="n">
-        <f aca="false">SUM('PR Plan'!$K$5:$K$19)</f>
-        <v>29.5</v>
+        <f aca="false">SUM('PR Plan'!$K$5:$K$20)</f>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2450,7 +2510,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>27.5</v>
       </c>
     </row>
@@ -2460,7 +2520,7 @@
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">IF(B9=0,0,B10/B9)</f>
-        <v>0.932203389830508</v>
+        <v>0.887096774193548</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2520,7 +2580,7 @@
         <v>8</v>
       </c>
       <c r="C18" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A18)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$L$5:$L$20,A18)</f>
         <v>8.5</v>
       </c>
       <c r="D18" s="11" t="n">
@@ -2528,7 +2588,7 @@
         <v>-0.5</v>
       </c>
       <c r="E18" s="12" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A18)</f>
+        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$20,A18)</f>
         <v>6</v>
       </c>
     </row>
@@ -2540,16 +2600,16 @@
         <v>12</v>
       </c>
       <c r="C19" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A19)</f>
-        <v>11.5</v>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$L$5:$L$20,A19)</f>
+        <v>13</v>
       </c>
       <c r="D19" s="11" t="n">
         <f aca="false">B19-C19</f>
-        <v>0.5</v>
+        <v>-1</v>
       </c>
       <c r="E19" s="12" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A19)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$20,A19)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2560,7 +2620,7 @@
         <v>5</v>
       </c>
       <c r="C20" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A20)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$L$5:$L$20,A20)</f>
         <v>8</v>
       </c>
       <c r="D20" s="11" t="n">
@@ -2568,7 +2628,7 @@
         <v>-3</v>
       </c>
       <c r="E20" s="12" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A20)</f>
+        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$20,A20)</f>
         <v>4</v>
       </c>
     </row>
@@ -2580,7 +2640,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$L$5:$L$19,A21)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$L$5:$L$20,A21)</f>
         <v>1.5</v>
       </c>
       <c r="D21" s="11" t="n">
@@ -2588,7 +2648,7 @@
         <v>-1.5</v>
       </c>
       <c r="E21" s="12" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$19,A21)</f>
+        <f aca="false">COUNTIF('PR Plan'!$L$5:$L$20,A21)</f>
         <v>1</v>
       </c>
     </row>
@@ -2602,15 +2662,15 @@
       </c>
       <c r="C22" s="14" t="n">
         <f aca="false">SUM(C18:C21)</f>
-        <v>29.5</v>
+        <v>31</v>
       </c>
       <c r="D22" s="14" t="n">
         <f aca="false">B22-C22</f>
-        <v>-4.5</v>
+        <v>-6</v>
       </c>
       <c r="E22" s="15" t="n">
         <f aca="false">SUM(E18:E21)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2642,15 +2702,15 @@
         <v>30</v>
       </c>
       <c r="B27" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A27)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A27)</f>
         <v>2.5</v>
       </c>
       <c r="C27" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A27)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A27)</f>
         <v>3</v>
       </c>
       <c r="D27" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A27,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A27,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>3</v>
       </c>
     </row>
@@ -2659,15 +2719,15 @@
         <v>31</v>
       </c>
       <c r="B28" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A28)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A28)</f>
         <v>3.5</v>
       </c>
       <c r="C28" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A28)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A28)</f>
         <v>2</v>
       </c>
       <c r="D28" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A28,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A28,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>2</v>
       </c>
     </row>
@@ -2676,15 +2736,15 @@
         <v>32</v>
       </c>
       <c r="B29" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A29)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A29)</f>
         <v>5</v>
       </c>
       <c r="C29" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A29)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A29)</f>
         <v>2</v>
       </c>
       <c r="D29" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A29,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A29,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>2</v>
       </c>
     </row>
@@ -2693,15 +2753,15 @@
         <v>33</v>
       </c>
       <c r="B30" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A30)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A30)</f>
         <v>3</v>
       </c>
       <c r="C30" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A30)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A30)</f>
         <v>1</v>
       </c>
       <c r="D30" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A30,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A30,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>1</v>
       </c>
     </row>
@@ -2710,15 +2770,15 @@
         <v>34</v>
       </c>
       <c r="B31" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A31)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A31)</f>
         <v>4</v>
       </c>
       <c r="C31" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A31)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A31)</f>
         <v>1</v>
       </c>
       <c r="D31" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A31,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A31,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>1</v>
       </c>
     </row>
@@ -2727,15 +2787,15 @@
         <v>35</v>
       </c>
       <c r="B32" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A32)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A32)</f>
         <v>8</v>
       </c>
       <c r="C32" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A32)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A32)</f>
         <v>4</v>
       </c>
       <c r="D32" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A32,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A32,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>4</v>
       </c>
     </row>
@@ -2744,15 +2804,15 @@
         <v>36</v>
       </c>
       <c r="B33" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A33)</f>
-        <v>1.5</v>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A33)</f>
+        <v>3</v>
       </c>
       <c r="C33" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A33)</f>
-        <v>1</v>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A33)</f>
+        <v>2</v>
       </c>
       <c r="D33" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A33,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A33,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>1</v>
       </c>
     </row>
@@ -2761,15 +2821,15 @@
         <v>37</v>
       </c>
       <c r="B34" s="11" t="n">
-        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$19,'PR Plan'!$D$5:$D$19,A34)</f>
+        <f aca="false">SUMIFS('PR Plan'!$K$5:$K$20,'PR Plan'!$D$5:$D$20,A34)</f>
         <v>2</v>
       </c>
       <c r="C34" s="18" t="n">
-        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$19,A34)</f>
+        <f aca="false">COUNTIF('PR Plan'!$D$5:$D$20,A34)</f>
         <v>1</v>
       </c>
       <c r="D34" s="18" t="n">
-        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$19,A34,'PR Plan'!$M$5:$M$19,"Done")</f>
+        <f aca="false">COUNTIFS('PR Plan'!$D$5:$D$20,A34,'PR Plan'!$M$5:$M$20,"Done")</f>
         <v>0</v>
       </c>
     </row>
@@ -2856,7 +2916,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -3650,39 +3710,87 @@
         <v>195</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="46" t="s">
+    <row r="20" customFormat="false" ht="174.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="32" t="s">
         <v>196</v>
       </c>
-      <c r="B20" s="47"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="47"/>
-      <c r="H20" s="47"/>
-      <c r="I20" s="47"/>
-      <c r="J20" s="47"/>
-      <c r="K20" s="48" t="n">
-        <f aca="false">SUM(K5:K19)</f>
-        <v>29.5</v>
-      </c>
-      <c r="L20" s="47"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="46" t="n">
-        <f aca="false">SUM(N5:N19)</f>
+      <c r="B20" s="33" t="s">
+        <v>197</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>198</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="35" t="s">
+        <v>163</v>
+      </c>
+      <c r="F20" s="33" t="s">
+        <v>199</v>
+      </c>
+      <c r="G20" s="33" t="s">
+        <v>200</v>
+      </c>
+      <c r="H20" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="I20" s="33" t="s">
+        <v>202</v>
+      </c>
+      <c r="J20" s="35" t="s">
+        <v>203</v>
+      </c>
+      <c r="K20" s="36" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L20" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="M20" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="N20" s="35" t="n">
+        <f aca="false">COUNTIF('Story Coverage'!$E:$E,A20)</f>
+        <v>0</v>
+      </c>
+      <c r="O20" s="38" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="46" t="s">
+        <v>206</v>
+      </c>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="47"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="47"/>
+      <c r="J21" s="47"/>
+      <c r="K21" s="48" t="n">
+        <f aca="false">SUM(K5:K20)</f>
+        <v>31</v>
+      </c>
+      <c r="L21" s="47"/>
+      <c r="M21" s="47"/>
+      <c r="N21" s="46" t="n">
+        <f aca="false">SUM(N5:N20)</f>
         <v>50</v>
       </c>
-      <c r="O20" s="47"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K21" s="16" t="s">
-        <v>197</v>
+      <c r="O21" s="47"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="K22" s="16" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:O19"/>
-  <conditionalFormatting sqref="M5:M19">
+  <conditionalFormatting sqref="M5:M20">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Done"</formula>
     </cfRule>
@@ -3696,7 +3804,7 @@
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E19">
+  <conditionalFormatting sqref="E5:E20">
     <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
       <formula>"Must"</formula>
     </cfRule>
@@ -3704,21 +3812,21 @@
       <formula>"Should"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:L19">
+  <conditionalFormatting sqref="A5:L20">
     <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="24">
       <formula>$M5="Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="M5:M20" type="list">
       <formula1>"Not started,In progress,In review,Done,Blocked"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E20" type="list">
       <formula1>"Must,Should,Could"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L19" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L20" type="list">
       <formula1>"Day 1 - Sun Oct 11,Day 2 - Mon Oct 12,Day 3 - Tue Oct 13 (AM),Stretch"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3754,49 +3862,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="D4" s="31" t="s">
         <v>58</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="H4" s="31" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="D5" s="35" t="s">
         <v>72</v>
@@ -3808,23 +3916,23 @@
         <v>119</v>
       </c>
       <c r="G5" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E5,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H5" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E5,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E5,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="D6" s="35" t="s">
         <v>72</v>
@@ -3836,23 +3944,23 @@
         <v>119</v>
       </c>
       <c r="G6" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E6,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H6" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E6,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E6,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>72</v>
@@ -3864,23 +3972,23 @@
         <v>119</v>
       </c>
       <c r="G7" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E7,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H7" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E7,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E7,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="D8" s="35" t="s">
         <v>72</v>
@@ -3890,49 +3998,49 @@
       </c>
       <c r="F8" s="35"/>
       <c r="G8" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E8,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H8" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E8,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E8,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="E9" s="35" t="s">
         <v>127</v>
       </c>
       <c r="F9" s="35"/>
       <c r="G9" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E9,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H9" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E9,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E9,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="D10" s="35" t="s">
         <v>72</v>
@@ -3942,23 +4050,23 @@
       </c>
       <c r="F10" s="35"/>
       <c r="G10" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E10,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H10" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E10,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E10,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="D11" s="35" t="s">
         <v>72</v>
@@ -3968,23 +4076,23 @@
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E11,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H11" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E11,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E11,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="D12" s="35" t="s">
         <v>72</v>
@@ -3994,23 +4102,23 @@
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E12,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H12" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E12,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E12,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="D13" s="35" t="s">
         <v>72</v>
@@ -4022,23 +4130,23 @@
         <v>111</v>
       </c>
       <c r="G13" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E13,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H13" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E13,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E13,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="D14" s="35" t="s">
         <v>72</v>
@@ -4048,23 +4156,23 @@
       </c>
       <c r="F14" s="35"/>
       <c r="G14" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E14,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H14" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E14,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E14,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="B15" s="33" t="s">
         <v>230</v>
       </c>
-      <c r="B15" s="33" t="s">
-        <v>220</v>
-      </c>
       <c r="C15" s="33" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="D15" s="35" t="s">
         <v>72</v>
@@ -4074,23 +4182,23 @@
       </c>
       <c r="F15" s="35"/>
       <c r="G15" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E15,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H15" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E15,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E15,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="D16" s="35" t="s">
         <v>72</v>
@@ -4099,26 +4207,26 @@
         <v>103</v>
       </c>
       <c r="F16" s="35" t="s">
-        <v>95</v>
+        <v>245</v>
       </c>
       <c r="G16" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E16,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E16,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H16" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E16,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E16,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="D17" s="35" t="s">
         <v>72</v>
@@ -4130,23 +4238,23 @@
         <v>127</v>
       </c>
       <c r="G17" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E17,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E17,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H17" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E17,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E17,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="D18" s="35" t="s">
         <v>72</v>
@@ -4158,23 +4266,23 @@
         <v>111</v>
       </c>
       <c r="G18" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E18,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E18,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H18" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E18,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E18,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="32" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="D19" s="35" t="s">
         <v>72</v>
@@ -4182,25 +4290,27 @@
       <c r="E19" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="35"/>
+      <c r="F19" s="35" t="s">
+        <v>196</v>
+      </c>
       <c r="G19" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E19,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E19,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H19" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E19,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E19,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="D20" s="35" t="s">
         <v>72</v>
@@ -4212,23 +4322,23 @@
         <v>127</v>
       </c>
       <c r="G20" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E20,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E20,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H20" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E20,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E20,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="D21" s="35" t="s">
         <v>72</v>
@@ -4238,23 +4348,23 @@
       </c>
       <c r="F21" s="35"/>
       <c r="G21" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E21,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E21,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H21" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E21,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E21,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="32" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="D22" s="35" t="s">
         <v>72</v>
@@ -4266,23 +4376,23 @@
         <v>79</v>
       </c>
       <c r="G22" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E22,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E22,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H22" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E22,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E22,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="32" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="D23" s="35" t="s">
         <v>72</v>
@@ -4294,23 +4404,23 @@
         <v>127</v>
       </c>
       <c r="G23" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E23,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E23,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H23" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E23,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E23,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="32" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="D24" s="35" t="s">
         <v>72</v>
@@ -4320,23 +4430,23 @@
       </c>
       <c r="F24" s="35"/>
       <c r="G24" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E24,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E24,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H24" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E24,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E24,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="32" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="D25" s="35" t="s">
         <v>72</v>
@@ -4348,23 +4458,23 @@
         <v>79</v>
       </c>
       <c r="G25" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E25,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E25,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H25" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E25,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E25,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="32" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="D26" s="35" t="s">
         <v>72</v>
@@ -4374,23 +4484,23 @@
       </c>
       <c r="F26" s="35"/>
       <c r="G26" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E26,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E26,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H26" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E26,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E26,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="32" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="D27" s="35" t="s">
         <v>72</v>
@@ -4402,23 +4512,23 @@
         <v>127</v>
       </c>
       <c r="G27" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E27,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E27,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H27" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E27,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E27,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="32" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="D28" s="35" t="s">
         <v>72</v>
@@ -4430,23 +4540,23 @@
         <v>111</v>
       </c>
       <c r="G28" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E28,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E28,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H28" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E28,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E28,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="32" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="D29" s="35" t="s">
         <v>72</v>
@@ -4458,23 +4568,23 @@
         <v>119</v>
       </c>
       <c r="G29" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E29,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H29" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E29,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E29,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="32" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="D30" s="35" t="s">
         <v>72</v>
@@ -4486,23 +4596,23 @@
         <v>95</v>
       </c>
       <c r="G30" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E30,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H30" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E30,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E30,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="32" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="D31" s="35" t="s">
         <v>72</v>
@@ -4514,23 +4624,23 @@
         <v>144</v>
       </c>
       <c r="G31" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E31,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E31,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H31" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E31,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E31,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="D32" s="35" t="s">
         <v>72</v>
@@ -4540,52 +4650,52 @@
       </c>
       <c r="F32" s="35"/>
       <c r="G32" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E32,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H32" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E32,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E32,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="32" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="E33" s="35" t="s">
         <v>144</v>
       </c>
       <c r="F33" s="35"/>
       <c r="G33" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E33,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H33" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E33,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E33,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="32" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="E34" s="35" t="s">
         <v>144</v>
@@ -4594,23 +4704,23 @@
         <v>103</v>
       </c>
       <c r="G34" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E34,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H34" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E34,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E34,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="32" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="D35" s="35" t="s">
         <v>72</v>
@@ -4620,23 +4730,23 @@
       </c>
       <c r="F35" s="35"/>
       <c r="G35" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E35,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H35" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E35,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E35,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="32" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="B36" s="33" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="D36" s="35" t="s">
         <v>72</v>
@@ -4646,23 +4756,23 @@
       </c>
       <c r="F36" s="35"/>
       <c r="G36" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E36,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H36" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E36,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E36,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="32" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="B37" s="33" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="C37" s="33" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="D37" s="35" t="s">
         <v>163</v>
@@ -4672,23 +4782,23 @@
       </c>
       <c r="F37" s="35"/>
       <c r="G37" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E37,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H37" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E37,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E37,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="32" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="B38" s="33" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="D38" s="35" t="s">
         <v>163</v>
@@ -4698,23 +4808,23 @@
       </c>
       <c r="F38" s="35"/>
       <c r="G38" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E38,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H38" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E38,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E38,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="32" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="B39" s="33" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="D39" s="35" t="s">
         <v>163</v>
@@ -4726,49 +4836,49 @@
         <v>111</v>
       </c>
       <c r="G39" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E39,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H39" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E39,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E39,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="32" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="B40" s="33" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="C40" s="33" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="E40" s="35" t="s">
         <v>160</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E40,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H40" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E40,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E40,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Stretch</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="32" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="D41" s="35" t="s">
         <v>163</v>
@@ -4780,23 +4890,23 @@
         <v>160</v>
       </c>
       <c r="G41" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E41,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H41" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E41,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E41,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="32" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="B42" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C42" s="33" t="s">
-        <v>294</v>
+        <v>305</v>
       </c>
       <c r="D42" s="35" t="s">
         <v>72</v>
@@ -4808,23 +4918,23 @@
         <v>169</v>
       </c>
       <c r="G42" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E42,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H42" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E42,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E42,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="32" t="s">
-        <v>295</v>
+        <v>306</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="D43" s="35" t="s">
         <v>72</v>
@@ -4834,23 +4944,23 @@
       </c>
       <c r="F43" s="35"/>
       <c r="G43" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E43,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E43,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H43" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E43,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E43,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="32" t="s">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="B44" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C44" s="33" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
       <c r="D44" s="35" t="s">
         <v>72</v>
@@ -4862,23 +4972,23 @@
         <v>169</v>
       </c>
       <c r="G44" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E44,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H44" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E44,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E44,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="32" t="s">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C45" s="33" t="s">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="D45" s="35" t="s">
         <v>72</v>
@@ -4888,23 +4998,23 @@
       </c>
       <c r="F45" s="35"/>
       <c r="G45" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E45,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E45,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H45" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E45,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E45,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="32" t="s">
-        <v>301</v>
+        <v>312</v>
       </c>
       <c r="B46" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C46" s="33" t="s">
-        <v>302</v>
+        <v>313</v>
       </c>
       <c r="D46" s="35" t="s">
         <v>72</v>
@@ -4914,23 +5024,23 @@
       </c>
       <c r="F46" s="35"/>
       <c r="G46" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E46,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E46,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H46" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E46,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E46,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="32" t="s">
-        <v>303</v>
+        <v>314</v>
       </c>
       <c r="B47" s="33" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="D47" s="35" t="s">
         <v>72</v>
@@ -4942,23 +5052,23 @@
         <v>169</v>
       </c>
       <c r="G47" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E47,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H47" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E47,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E47,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="32" t="s">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="B48" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C48" s="33" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="D48" s="35" t="s">
         <v>72</v>
@@ -4970,23 +5080,23 @@
         <v>69</v>
       </c>
       <c r="G48" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E48,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H48" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E48,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E48,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="32" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="B49" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C49" s="33" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
       <c r="D49" s="35" t="s">
         <v>72</v>
@@ -4996,23 +5106,23 @@
       </c>
       <c r="F49" s="35"/>
       <c r="G49" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E49,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E49,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H49" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E49,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E49,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="32" t="s">
-        <v>310</v>
+        <v>321</v>
       </c>
       <c r="B50" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C50" s="33" t="s">
-        <v>311</v>
+        <v>322</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>72</v>
@@ -5022,23 +5132,23 @@
       </c>
       <c r="F50" s="35"/>
       <c r="G50" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E50,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E50,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H50" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E50,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E50,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 2 - Mon Oct 12</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="32" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="B51" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="D51" s="35" t="s">
         <v>72</v>
@@ -5047,26 +5157,26 @@
         <v>111</v>
       </c>
       <c r="F51" s="35" t="s">
-        <v>169</v>
+        <v>325</v>
       </c>
       <c r="G51" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E51,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H51" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E51,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E51,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="32" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="B52" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C52" s="33" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="D52" s="35" t="s">
         <v>163</v>
@@ -5076,49 +5186,49 @@
       </c>
       <c r="F52" s="35"/>
       <c r="G52" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E52,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E52,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H52" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E52,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E52,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 1 - Sun Oct 11</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="32" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="B53" s="33" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="C53" s="33" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="D53" s="35" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="E53" s="35" t="s">
         <v>169</v>
       </c>
       <c r="F53" s="35"/>
       <c r="G53" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E53,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H53" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E53,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E53,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="32" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B54" s="33" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="C54" s="33" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="D54" s="35" t="s">
         <v>163</v>
@@ -5130,11 +5240,11 @@
         <v>144</v>
       </c>
       <c r="G54" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$M$5:$M$20,MATCH(E54,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Done</v>
       </c>
       <c r="H54" s="49" t="str">
-        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$19,MATCH(E54,'PR Plan'!$A$5:$A$19,0)),"-")</f>
+        <f aca="false">IFERROR(INDEX('PR Plan'!$L$5:$L$20,MATCH(E54,'PR Plan'!$A$5:$A$20,0)),"-")</f>
         <v>Day 3 - Tue Oct 13 (AM)</v>
       </c>
     </row>
@@ -5175,7 +5285,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -5189,55 +5299,55 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="G5" s="35" t="s">
         <v>119</v>
@@ -5245,22 +5355,22 @@
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="G6" s="35" t="s">
         <v>111</v>
@@ -5268,22 +5378,22 @@
     </row>
     <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="B7" s="35" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="G7" s="35" t="s">
         <v>103</v>
@@ -5291,22 +5401,22 @@
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="B8" s="35" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="G8" s="35" t="s">
         <v>95</v>
@@ -5314,22 +5424,22 @@
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="G9" s="35" t="s">
         <v>79</v>
@@ -5337,22 +5447,22 @@
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="C10" s="50" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="G10" s="35" t="s">
         <v>119</v>
@@ -5360,22 +5470,22 @@
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B11" s="35" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="50" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="E11" s="33" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="G11" s="35" t="s">
         <v>135</v>
@@ -5383,22 +5493,22 @@
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="E12" s="33" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="G12" s="35" t="s">
         <v>111</v>
@@ -5406,22 +5516,22 @@
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="B13" s="35" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="G13" s="35" t="s">
         <v>111</v>
@@ -5429,22 +5539,22 @@
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="C14" s="50" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="E14" s="33" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="G14" s="35" t="s">
         <v>79</v>
@@ -5452,22 +5562,22 @@
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="B15" s="35" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="C15" s="50" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="G15" s="35" t="s">
         <v>79</v>
@@ -5475,22 +5585,22 @@
     </row>
     <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="C16" s="50" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="G16" s="35" t="s">
         <v>69</v>
@@ -5498,22 +5608,22 @@
     </row>
     <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="32" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="C17" s="50" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="G17" s="35" t="s">
         <v>103</v>
@@ -5521,25 +5631,48 @@
     </row>
     <row r="18" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="32" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="B18" s="35" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="C18" s="50" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="F18" s="33" t="s">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="G18" s="35" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="32" t="s">
+        <v>424</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>425</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>426</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>427</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>428</v>
+      </c>
+      <c r="F19" s="33" t="s">
+        <v>429</v>
+      </c>
+      <c r="G19" s="35" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>